<commit_message>
Score rep 2 of the blind skeleton drill
Second attempt scores 72/78, up from 57/78. All four supporting
schedules, period headers, subtotals, a balance check row and a working
revolver block are now present; the income statement and schedules
blocks are complete.

Adds a Rep 2 Notes tab recording nine findings, chief among them an
uncapped revolver repayment that drives the balance negative whenever
excess cash exceeds the amount outstanding, plus a live stress table
contrasting the formula written against the correct MIN/MAX form.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UX5HPwj2AEakAb4LMEQ7Bv
</commit_message>
<xml_diff>
--- a/learning/model-practice/Day_2_scorecard_and_ladder.xlsx
+++ b/learning/model-practice/Day_2_scorecard_and_ladder.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Skeleton Scorecard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Day 2 Build" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Ladder" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Rep 2 Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Day 2 Build" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Ladder" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -113,6 +114,30 @@
       <color rgb="FF7F7F7F"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF008000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFC00000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -173,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -226,6 +251,28 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -591,7 +638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K104"/>
+  <dimension ref="B2:K104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -607,7 +654,6 @@
     <col width="8" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -629,7 +675,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -702,7 +747,6 @@
         <v/>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="B9" s="6" t="inlineStr">
         <is>
@@ -784,7 +828,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F11" s="13" t="n"/>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G11" s="13" t="n"/>
       <c r="H11" s="13" t="n"/>
       <c r="I11" s="13" t="n"/>
@@ -804,7 +852,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F12" s="13" t="n"/>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G12" s="13" t="n"/>
       <c r="H12" s="13" t="n"/>
       <c r="I12" s="13" t="n"/>
@@ -824,7 +876,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F13" s="13" t="n"/>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G13" s="13" t="n"/>
       <c r="H13" s="13" t="n"/>
       <c r="I13" s="13" t="n"/>
@@ -844,7 +900,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F14" s="13" t="n"/>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G14" s="13" t="n"/>
       <c r="H14" s="13" t="n"/>
       <c r="I14" s="13" t="n"/>
@@ -868,7 +928,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F15" s="13" t="n"/>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G15" s="13" t="n"/>
       <c r="H15" s="13" t="n"/>
       <c r="I15" s="13" t="n"/>
@@ -888,7 +952,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F16" s="13" t="n"/>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G16" s="13" t="n"/>
       <c r="H16" s="13" t="n"/>
       <c r="I16" s="13" t="n"/>
@@ -908,7 +976,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F17" s="13" t="n"/>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G17" s="13" t="n"/>
       <c r="H17" s="13" t="n"/>
       <c r="I17" s="13" t="n"/>
@@ -928,7 +1000,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F18" s="13" t="n"/>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G18" s="13" t="n"/>
       <c r="H18" s="13" t="n"/>
       <c r="I18" s="13" t="n"/>
@@ -948,7 +1024,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F19" s="13" t="n"/>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G19" s="13" t="n"/>
       <c r="H19" s="13" t="n"/>
       <c r="I19" s="13" t="n"/>
@@ -972,7 +1052,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F20" s="13" t="n"/>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G20" s="13" t="n"/>
       <c r="H20" s="13" t="n"/>
       <c r="I20" s="13" t="n"/>
@@ -992,7 +1076,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F21" s="13" t="n"/>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="G21" s="13" t="n"/>
       <c r="H21" s="13" t="n"/>
       <c r="I21" s="13" t="n"/>
@@ -1012,7 +1100,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F22" s="13" t="n"/>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G22" s="13" t="n"/>
       <c r="H22" s="13" t="n"/>
       <c r="I22" s="13" t="n"/>
@@ -1036,7 +1128,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F23" s="13" t="n"/>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G23" s="13" t="n"/>
       <c r="H23" s="13" t="n"/>
       <c r="I23" s="13" t="n"/>
@@ -1060,7 +1156,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F24" s="13" t="n"/>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G24" s="13" t="n"/>
       <c r="H24" s="13" t="n"/>
       <c r="I24" s="13" t="n"/>
@@ -1084,7 +1184,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F25" s="13" t="n"/>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="G25" s="13" t="n"/>
       <c r="H25" s="13" t="n"/>
       <c r="I25" s="13" t="n"/>
@@ -1104,7 +1208,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F26" s="13" t="n"/>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G26" s="13" t="n"/>
       <c r="H26" s="13" t="n"/>
       <c r="I26" s="13" t="n"/>
@@ -1124,7 +1232,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F27" s="13" t="n"/>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G27" s="13" t="n"/>
       <c r="H27" s="13" t="n"/>
       <c r="I27" s="13" t="n"/>
@@ -1144,7 +1256,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F28" s="13" t="n"/>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G28" s="13" t="n"/>
       <c r="H28" s="13" t="n"/>
       <c r="I28" s="13" t="n"/>
@@ -1180,7 +1296,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F30" s="13" t="n"/>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G30" s="13" t="n"/>
       <c r="H30" s="13" t="n"/>
       <c r="I30" s="13" t="n"/>
@@ -1200,7 +1320,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F31" s="13" t="n"/>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G31" s="13" t="n"/>
       <c r="H31" s="13" t="n"/>
       <c r="I31" s="13" t="n"/>
@@ -1224,7 +1348,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F32" s="13" t="n"/>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G32" s="13" t="n"/>
       <c r="H32" s="13" t="n"/>
       <c r="I32" s="13" t="n"/>
@@ -1244,7 +1372,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F33" s="13" t="n"/>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G33" s="13" t="n"/>
       <c r="H33" s="13" t="n"/>
       <c r="I33" s="13" t="n"/>
@@ -1264,7 +1396,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F34" s="13" t="n"/>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G34" s="13" t="n"/>
       <c r="H34" s="13" t="n"/>
       <c r="I34" s="13" t="n"/>
@@ -1284,7 +1420,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F35" s="13" t="n"/>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G35" s="13" t="n"/>
       <c r="H35" s="13" t="n"/>
       <c r="I35" s="13" t="n"/>
@@ -1304,7 +1444,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F36" s="13" t="n"/>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G36" s="13" t="n"/>
       <c r="H36" s="13" t="n"/>
       <c r="I36" s="13" t="n"/>
@@ -1324,7 +1468,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F37" s="13" t="n"/>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G37" s="13" t="n"/>
       <c r="H37" s="13" t="n"/>
       <c r="I37" s="13" t="n"/>
@@ -1348,7 +1496,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F38" s="13" t="n"/>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G38" s="13" t="n"/>
       <c r="H38" s="13" t="n"/>
       <c r="I38" s="13" t="n"/>
@@ -1368,7 +1520,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F39" s="13" t="n"/>
+      <c r="F39" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G39" s="13" t="n"/>
       <c r="H39" s="13" t="n"/>
       <c r="I39" s="13" t="n"/>
@@ -1388,7 +1544,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F40" s="13" t="n"/>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G40" s="13" t="n"/>
       <c r="H40" s="13" t="n"/>
       <c r="I40" s="13" t="n"/>
@@ -1408,7 +1568,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F41" s="13" t="n"/>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G41" s="13" t="n"/>
       <c r="H41" s="13" t="n"/>
       <c r="I41" s="13" t="n"/>
@@ -1428,7 +1592,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F42" s="13" t="n"/>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G42" s="13" t="n"/>
       <c r="H42" s="13" t="n"/>
       <c r="I42" s="13" t="n"/>
@@ -1448,7 +1616,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F43" s="13" t="n"/>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G43" s="13" t="n"/>
       <c r="H43" s="13" t="n"/>
       <c r="I43" s="13" t="n"/>
@@ -1484,7 +1656,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F45" s="13" t="n"/>
+      <c r="F45" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G45" s="13" t="n"/>
       <c r="H45" s="13" t="n"/>
       <c r="I45" s="13" t="n"/>
@@ -1504,7 +1680,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F46" s="13" t="n"/>
+      <c r="F46" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G46" s="13" t="n"/>
       <c r="H46" s="13" t="n"/>
       <c r="I46" s="13" t="n"/>
@@ -1524,7 +1704,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F47" s="13" t="n"/>
+      <c r="F47" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G47" s="13" t="n"/>
       <c r="H47" s="13" t="n"/>
       <c r="I47" s="13" t="n"/>
@@ -1548,7 +1732,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F48" s="13" t="n"/>
+      <c r="F48" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G48" s="13" t="n"/>
       <c r="H48" s="13" t="n"/>
       <c r="I48" s="13" t="n"/>
@@ -1568,7 +1756,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F49" s="13" t="n"/>
+      <c r="F49" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G49" s="13" t="n"/>
       <c r="H49" s="13" t="n"/>
       <c r="I49" s="13" t="n"/>
@@ -1588,7 +1780,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F50" s="13" t="n"/>
+      <c r="F50" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G50" s="13" t="n"/>
       <c r="H50" s="13" t="n"/>
       <c r="I50" s="13" t="n"/>
@@ -1608,7 +1804,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F51" s="13" t="n"/>
+      <c r="F51" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G51" s="13" t="n"/>
       <c r="H51" s="13" t="n"/>
       <c r="I51" s="13" t="n"/>
@@ -1628,7 +1828,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F52" s="13" t="n"/>
+      <c r="F52" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G52" s="13" t="n"/>
       <c r="H52" s="13" t="n"/>
       <c r="I52" s="13" t="n"/>
@@ -1648,7 +1852,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F53" s="13" t="n"/>
+      <c r="F53" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G53" s="13" t="n"/>
       <c r="H53" s="13" t="n"/>
       <c r="I53" s="13" t="n"/>
@@ -1672,7 +1880,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F54" s="13" t="n"/>
+      <c r="F54" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="G54" s="13" t="n"/>
       <c r="H54" s="13" t="n"/>
       <c r="I54" s="13" t="n"/>
@@ -1692,7 +1904,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F55" s="13" t="n"/>
+      <c r="F55" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G55" s="13" t="n"/>
       <c r="H55" s="13" t="n"/>
       <c r="I55" s="13" t="n"/>
@@ -1712,7 +1928,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F56" s="13" t="n"/>
+      <c r="F56" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G56" s="13" t="n"/>
       <c r="H56" s="13" t="n"/>
       <c r="I56" s="13" t="n"/>
@@ -1736,7 +1956,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F57" s="13" t="n"/>
+      <c r="F57" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G57" s="13" t="n"/>
       <c r="H57" s="13" t="n"/>
       <c r="I57" s="13" t="n"/>
@@ -1756,7 +1980,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F58" s="13" t="n"/>
+      <c r="F58" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G58" s="13" t="n"/>
       <c r="H58" s="13" t="n"/>
       <c r="I58" s="13" t="n"/>
@@ -1776,7 +2004,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F59" s="13" t="n"/>
+      <c r="F59" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G59" s="13" t="n"/>
       <c r="H59" s="13" t="n"/>
       <c r="I59" s="13" t="n"/>
@@ -1796,7 +2028,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F60" s="13" t="n"/>
+      <c r="F60" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G60" s="13" t="n"/>
       <c r="H60" s="13" t="n"/>
       <c r="I60" s="13" t="n"/>
@@ -1816,7 +2052,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F61" s="13" t="n"/>
+      <c r="F61" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G61" s="13" t="n"/>
       <c r="H61" s="13" t="n"/>
       <c r="I61" s="13" t="n"/>
@@ -1836,7 +2076,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F62" s="13" t="n"/>
+      <c r="F62" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G62" s="13" t="n"/>
       <c r="H62" s="13" t="n"/>
       <c r="I62" s="13" t="n"/>
@@ -1856,7 +2100,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F63" s="13" t="n"/>
+      <c r="F63" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G63" s="13" t="n"/>
       <c r="H63" s="13" t="n"/>
       <c r="I63" s="13" t="n"/>
@@ -1880,7 +2128,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F64" s="13" t="n"/>
+      <c r="F64" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G64" s="13" t="n"/>
       <c r="H64" s="13" t="n"/>
       <c r="I64" s="13" t="n"/>
@@ -1916,7 +2168,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F66" s="13" t="n"/>
+      <c r="F66" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G66" s="13" t="n"/>
       <c r="H66" s="13" t="n"/>
       <c r="I66" s="13" t="n"/>
@@ -1936,7 +2192,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F67" s="13" t="n"/>
+      <c r="F67" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G67" s="13" t="n"/>
       <c r="H67" s="13" t="n"/>
       <c r="I67" s="13" t="n"/>
@@ -1956,7 +2216,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F68" s="13" t="n"/>
+      <c r="F68" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G68" s="13" t="n"/>
       <c r="H68" s="13" t="n"/>
       <c r="I68" s="13" t="n"/>
@@ -1976,7 +2240,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F69" s="13" t="n"/>
+      <c r="F69" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G69" s="13" t="n"/>
       <c r="H69" s="13" t="n"/>
       <c r="I69" s="13" t="n"/>
@@ -1996,7 +2264,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F70" s="13" t="n"/>
+      <c r="F70" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G70" s="13" t="n"/>
       <c r="H70" s="13" t="n"/>
       <c r="I70" s="13" t="n"/>
@@ -2016,7 +2288,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F71" s="13" t="n"/>
+      <c r="F71" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G71" s="13" t="n"/>
       <c r="H71" s="13" t="n"/>
       <c r="I71" s="13" t="n"/>
@@ -2036,7 +2312,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F72" s="13" t="n"/>
+      <c r="F72" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G72" s="13" t="n"/>
       <c r="H72" s="13" t="n"/>
       <c r="I72" s="13" t="n"/>
@@ -2056,7 +2336,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F73" s="13" t="n"/>
+      <c r="F73" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G73" s="13" t="n"/>
       <c r="H73" s="13" t="n"/>
       <c r="I73" s="13" t="n"/>
@@ -2076,7 +2360,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F74" s="13" t="n"/>
+      <c r="F74" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G74" s="13" t="n"/>
       <c r="H74" s="13" t="n"/>
       <c r="I74" s="13" t="n"/>
@@ -2096,7 +2384,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F75" s="13" t="n"/>
+      <c r="F75" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G75" s="13" t="n"/>
       <c r="H75" s="13" t="n"/>
       <c r="I75" s="13" t="n"/>
@@ -2116,7 +2408,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F76" s="13" t="n"/>
+      <c r="F76" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="G76" s="13" t="n"/>
       <c r="H76" s="13" t="n"/>
       <c r="I76" s="13" t="n"/>
@@ -2136,7 +2432,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F77" s="13" t="n"/>
+      <c r="F77" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G77" s="13" t="n"/>
       <c r="H77" s="13" t="n"/>
       <c r="I77" s="13" t="n"/>
@@ -2160,7 +2460,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F78" s="13" t="n"/>
+      <c r="F78" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G78" s="13" t="n"/>
       <c r="H78" s="13" t="n"/>
       <c r="I78" s="13" t="n"/>
@@ -2180,7 +2484,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F79" s="13" t="n"/>
+      <c r="F79" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G79" s="13" t="n"/>
       <c r="H79" s="13" t="n"/>
       <c r="I79" s="13" t="n"/>
@@ -2200,7 +2508,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F80" s="13" t="n"/>
+      <c r="F80" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G80" s="13" t="n"/>
       <c r="H80" s="13" t="n"/>
       <c r="I80" s="13" t="n"/>
@@ -2220,7 +2532,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F81" s="13" t="n"/>
+      <c r="F81" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G81" s="13" t="n"/>
       <c r="H81" s="13" t="n"/>
       <c r="I81" s="13" t="n"/>
@@ -2240,7 +2556,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F82" s="13" t="n"/>
+      <c r="F82" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G82" s="13" t="n"/>
       <c r="H82" s="13" t="n"/>
       <c r="I82" s="13" t="n"/>
@@ -2280,7 +2600,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F84" s="13" t="n"/>
+      <c r="F84" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G84" s="13" t="n"/>
       <c r="H84" s="13" t="n"/>
       <c r="I84" s="13" t="n"/>
@@ -2300,7 +2624,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F85" s="13" t="n"/>
+      <c r="F85" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G85" s="13" t="n"/>
       <c r="H85" s="13" t="n"/>
       <c r="I85" s="13" t="n"/>
@@ -2320,7 +2648,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F86" s="13" t="n"/>
+      <c r="F86" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G86" s="13" t="n"/>
       <c r="H86" s="13" t="n"/>
       <c r="I86" s="13" t="n"/>
@@ -2340,7 +2672,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F87" s="13" t="n"/>
+      <c r="F87" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G87" s="13" t="n"/>
       <c r="H87" s="13" t="n"/>
       <c r="I87" s="13" t="n"/>
@@ -2360,7 +2696,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F88" s="13" t="n"/>
+      <c r="F88" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G88" s="13" t="n"/>
       <c r="H88" s="13" t="n"/>
       <c r="I88" s="13" t="n"/>
@@ -2400,7 +2740,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F90" s="13" t="n"/>
+      <c r="F90" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G90" s="13" t="n"/>
       <c r="H90" s="13" t="n"/>
       <c r="I90" s="13" t="n"/>
@@ -2420,7 +2764,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F91" s="13" t="n"/>
+      <c r="F91" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="G91" s="13" t="n"/>
       <c r="H91" s="13" t="n"/>
       <c r="I91" s="13" t="n"/>
@@ -2440,7 +2788,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F92" s="13" t="n"/>
+      <c r="F92" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="G92" s="13" t="n"/>
       <c r="H92" s="13" t="n"/>
       <c r="I92" s="13" t="n"/>
@@ -2460,7 +2812,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="F93" s="13" t="n"/>
+      <c r="F93" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="G93" s="13" t="n"/>
       <c r="H93" s="13" t="n"/>
       <c r="I93" s="13" t="n"/>
@@ -2851,6 +3207,502 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:H25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="78" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Rep 2 Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="32" t="inlineStr">
+        <is>
+          <t>Scored 72 / 78. Up from 57 / 78 on rep 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Every structural gap from rep 1 closed except one. What follows is what is left, ranked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Finding</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Why it matters</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>Revolver repayment has no cap</t>
+        </is>
+      </c>
+      <c r="E8" s="30">
+        <f>IF(D181&gt;D180,(D181-D180),0) repays the full excess over minimum cash, even when you owe less than that. The revolver goes negative. Your test numbers (cash 70, min 50, owed 20) are the one case where excess exactly equals the balance, so it could not show. Fix: =MIN(beginning balance, MAX(0, cash - minimum)).</f>
+        <v/>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>Drill 3 on the drills page. This is precisely the cap it exists to teach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C9" s="35" t="inlineStr">
+        <is>
+          <t>WIRING</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>Revolver reads final cash, not cash before the revolver</t>
+        </is>
+      </c>
+      <c r="E9" s="30" t="inlineStr">
+        <is>
+          <t>D181 links to the balance sheet cash line. That line is the OUTPUT of the sweep, so once you add numbers this becomes circular in the wrong way. It must reference cash before any revolver activity: opening cash + CFO + CFI + financing excluding the revolver.</t>
+        </is>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>Bites on Day 6 when the model first closes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="inlineStr">
+        <is>
+          <t>MISS</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>Income taxes payable is still absent from the balance sheet</t>
+        </is>
+      </c>
+      <c r="E10" s="30" t="inlineStr">
+        <is>
+          <t>You have the days assumption (B14), the working capital schedule line (B128) and the cash flow line (B102) - but no balance in current liabilities. Same miss as rep 1. A line that flows through the CFS must have a home on the BS.</t>
+        </is>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>This is your one repeat error. Put it on the next rep's checklist first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>WRONG PLACE</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>'Dividends' sits as a line inside shareholders' equity</t>
+        </is>
+      </c>
+      <c r="E11" s="30" t="inlineStr">
+        <is>
+          <t>B82. Dividends are a flow, not a balance. They belong on the income statement, in financing on the cash flow statement, and as a deduction inside the equity roll-forward - not as a standing balance sheet row.</t>
+        </is>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>Delete the row; the equity schedule already handles it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C12" s="35" t="inlineStr">
+        <is>
+          <t>SLIP</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>No effective tax rate assumption</t>
+        </is>
+      </c>
+      <c r="E12" s="30" t="inlineStr">
+        <is>
+          <t>B15 reads 'Effective interest rate', sitting directly above three other interest rate lines. You have a Taxes line on the income statement and an income-tax-payable days driver, so the tax rate is what that row was meant to be.</t>
+        </is>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>Almost certainly a typing slip rather than a recall failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C13" s="35" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>No revolver line in cash flow financing</t>
+        </is>
+      </c>
+      <c r="E13" s="30" t="inlineStr">
+        <is>
+          <t>The financing section has debt, equity and dividends. The revolver draw and repayment need their own line there so the sweep actually moves cash.</t>
+        </is>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>Minor - you built the schedule, it just is not wired to the CFS yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C14" s="35" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>No mandatory debt amortisation</t>
+        </is>
+      </c>
+      <c r="E14" s="30" t="inlineStr">
+        <is>
+          <t>The debt schedule is beginning + issuance = ending. A real one also has the scheduled repayment as its own line.</t>
+        </is>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>Add on Day 8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C15" s="35" t="inlineStr">
+        <is>
+          <t>STRUCTURE</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>No colour convention anywhere</t>
+        </is>
+      </c>
+      <c r="E15" s="30" t="inlineStr">
+        <is>
+          <t>Every cell in the file uses the default theme font. Blue for hardcoded inputs, black for formulas, green for cross-sheet links. Start this now, while the model is small enough that it costs nothing.</t>
+        </is>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>Also: mark which periods are actual and which are projected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="58" customHeight="1">
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C16" s="35" t="inlineStr">
+        <is>
+          <t>NIT</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>Cash from Operations header sits below net income</t>
+        </is>
+      </c>
+      <c r="E16" s="30" t="inlineStr">
+        <is>
+          <t>B98 is a section header but it appears after net income and depreciation. Move it above B95 so the section reads top-down.</t>
+        </is>
+      </c>
+      <c r="F16" s="34" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>WHY THE REVOLVER FORMULA FAILS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="36" t="inlineStr">
+        <is>
+          <t>Edit the blue cells - the two columns disagree whenever excess cash exceeds what you owe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="37" t="inlineStr">
+        <is>
+          <t>Beginning</t>
+        </is>
+      </c>
+      <c r="C20" s="37" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="D20" s="37" t="inlineStr">
+        <is>
+          <t>Min cash</t>
+        </is>
+      </c>
+      <c r="E20" s="37" t="inlineStr">
+        <is>
+          <t>Yours: repay</t>
+        </is>
+      </c>
+      <c r="F20" s="37" t="inlineStr">
+        <is>
+          <t>Yours: ending</t>
+        </is>
+      </c>
+      <c r="G20" s="37" t="inlineStr">
+        <is>
+          <t>Correct: repay</t>
+        </is>
+      </c>
+      <c r="H20" s="37" t="inlineStr">
+        <is>
+          <t>Correct: ending</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="38" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="38" t="n">
+        <v>70</v>
+      </c>
+      <c r="D21" s="38" t="n">
+        <v>50</v>
+      </c>
+      <c r="E21" s="39">
+        <f>IF(C21&gt;D21,(C21-D21),0)</f>
+        <v/>
+      </c>
+      <c r="F21" s="40">
+        <f>B21-E21</f>
+        <v/>
+      </c>
+      <c r="G21" s="39">
+        <f>MIN(B21,MAX(0,C21-D21))</f>
+        <v/>
+      </c>
+      <c r="H21" s="41">
+        <f>B21-G21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="38" t="n">
+        <v>20</v>
+      </c>
+      <c r="C22" s="38" t="n">
+        <v>100</v>
+      </c>
+      <c r="D22" s="38" t="n">
+        <v>50</v>
+      </c>
+      <c r="E22" s="39">
+        <f>IF(C22&gt;D22,(C22-D22),0)</f>
+        <v/>
+      </c>
+      <c r="F22" s="40">
+        <f>B22-E22</f>
+        <v/>
+      </c>
+      <c r="G22" s="39">
+        <f>MIN(B22,MAX(0,C22-D22))</f>
+        <v/>
+      </c>
+      <c r="H22" s="41">
+        <f>B22-G22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="38" t="n">
+        <v>120</v>
+      </c>
+      <c r="D23" s="38" t="n">
+        <v>50</v>
+      </c>
+      <c r="E23" s="39">
+        <f>IF(C23&gt;D23,(C23-D23),0)</f>
+        <v/>
+      </c>
+      <c r="F23" s="40">
+        <f>B23-E23</f>
+        <v/>
+      </c>
+      <c r="G23" s="39">
+        <f>MIN(B23,MAX(0,C23-D23))</f>
+        <v/>
+      </c>
+      <c r="H23" s="41">
+        <f>B23-G23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="38" t="n">
+        <v>10</v>
+      </c>
+      <c r="C24" s="38" t="n">
+        <v>200</v>
+      </c>
+      <c r="D24" s="38" t="n">
+        <v>50</v>
+      </c>
+      <c r="E24" s="39">
+        <f>IF(C24&gt;D24,(C24-D24),0)</f>
+        <v/>
+      </c>
+      <c r="F24" s="40">
+        <f>B24-E24</f>
+        <v/>
+      </c>
+      <c r="G24" s="39">
+        <f>MIN(B24,MAX(0,C24-D24))</f>
+        <v/>
+      </c>
+      <c r="H24" s="41">
+        <f>B24-G24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="38" t="n">
+        <v>20</v>
+      </c>
+      <c r="C25" s="38" t="n">
+        <v>30</v>
+      </c>
+      <c r="D25" s="38" t="n">
+        <v>50</v>
+      </c>
+      <c r="E25" s="39">
+        <f>IF(C25&gt;D25,(C25-D25),0)</f>
+        <v/>
+      </c>
+      <c r="F25" s="40">
+        <f>B25-E25</f>
+        <v/>
+      </c>
+      <c r="G25" s="39">
+        <f>MIN(B25,MAX(0,C25-D25))</f>
+        <v/>
+      </c>
+      <c r="H25" s="41">
+        <f>B25-G25</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3023,13 +3875,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E26"/>
+  <dimension ref="B2:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -3104,13 +3956,17 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="42" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="C9" s="29" t="inlineStr"/>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="D9" s="17" t="inlineStr">
         <is>
           <t>Periods + assumptions</t>
@@ -3118,7 +3974,7 @@
       </c>
       <c r="E9" s="30" t="inlineStr">
         <is>
-          <t>Skeleton from blank, then add the period columns and every assumption with a real value. Blue text for all of them. Stop there.</t>
+          <t>Skeleton rebuilt at 72/78 with all four schedules and a working revolver block. Periods, subtotals and balance check added. Next: fix the six findings, then add assumption values.</t>
         </is>
       </c>
     </row>
@@ -3338,6 +4194,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="B23" s="23" t="inlineStr">
         <is>
@@ -3366,6 +4223,9 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Score rep 3 of the blind skeleton drill
Third attempt scores 71/78 in 44 minutes, essentially flat against rep 2
but with a meaningful reshuffle underneath: the balance sheet is now
complete at 20/20 with income taxes payable and the effective tax rate
both corrected, while the revolver block and its two assumptions were
lost after being present last rep.

Replaces the per-rep notes tab with a rolling Findings Log that carries
each finding across reps with a status, so fixes and regressions stay
visible over time. Adds a minutes row to the scorecard.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UX5HPwj2AEakAb4LMEQ7Bv
</commit_message>
<xml_diff>
--- a/learning/model-practice/Day_2_scorecard_and_ladder.xlsx
+++ b/learning/model-practice/Day_2_scorecard_and_ladder.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Skeleton Scorecard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Rep 2 Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Findings Log" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Day 2 Build" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Ladder" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -138,6 +138,35 @@
       <color rgb="FFFFFFFF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFB26B00"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF008000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFB26B00"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFB26B00"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -198,7 +227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -273,6 +302,13 @@
     <xf numFmtId="3" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -747,6 +783,23 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Minutes</t>
+        </is>
+      </c>
+      <c r="D8" s="36" t="inlineStr">
+        <is>
+          <t>Target: under 15 for a labels-only skeleton</t>
+        </is>
+      </c>
+      <c r="E8" s="42" t="n"/>
+      <c r="F8" s="42" t="n"/>
+      <c r="G8" s="42" t="n">
+        <v>44</v>
+      </c>
+    </row>
     <row r="9">
       <c r="B9" s="6" t="inlineStr">
         <is>
@@ -833,7 +886,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G11" s="13" t="n"/>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H11" s="13" t="n"/>
       <c r="I11" s="13" t="n"/>
       <c r="J11" s="13" t="n"/>
@@ -857,7 +914,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G12" s="13" t="n"/>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H12" s="13" t="n"/>
       <c r="I12" s="13" t="n"/>
       <c r="J12" s="13" t="n"/>
@@ -881,7 +942,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G13" s="13" t="n"/>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H13" s="13" t="n"/>
       <c r="I13" s="13" t="n"/>
       <c r="J13" s="13" t="n"/>
@@ -905,7 +970,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G14" s="13" t="n"/>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H14" s="13" t="n"/>
       <c r="I14" s="13" t="n"/>
       <c r="J14" s="13" t="n"/>
@@ -933,7 +1002,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G15" s="13" t="n"/>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H15" s="13" t="n"/>
       <c r="I15" s="13" t="n"/>
       <c r="J15" s="13" t="n"/>
@@ -957,7 +1030,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G16" s="13" t="n"/>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H16" s="13" t="n"/>
       <c r="I16" s="13" t="n"/>
       <c r="J16" s="13" t="n"/>
@@ -981,7 +1058,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n"/>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H17" s="13" t="n"/>
       <c r="I17" s="13" t="n"/>
       <c r="J17" s="13" t="n"/>
@@ -1005,7 +1086,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G18" s="13" t="n"/>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H18" s="13" t="n"/>
       <c r="I18" s="13" t="n"/>
       <c r="J18" s="13" t="n"/>
@@ -1029,7 +1114,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G19" s="13" t="n"/>
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H19" s="13" t="n"/>
       <c r="I19" s="13" t="n"/>
       <c r="J19" s="13" t="n"/>
@@ -1057,7 +1146,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G20" s="13" t="n"/>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H20" s="13" t="n"/>
       <c r="I20" s="13" t="n"/>
       <c r="J20" s="13" t="n"/>
@@ -1081,7 +1174,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G21" s="13" t="n"/>
+      <c r="G21" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H21" s="13" t="n"/>
       <c r="I21" s="13" t="n"/>
       <c r="J21" s="13" t="n"/>
@@ -1105,7 +1202,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G22" s="13" t="n"/>
+      <c r="G22" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H22" s="13" t="n"/>
       <c r="I22" s="13" t="n"/>
       <c r="J22" s="13" t="n"/>
@@ -1133,7 +1234,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G23" s="13" t="n"/>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="H23" s="13" t="n"/>
       <c r="I23" s="13" t="n"/>
       <c r="J23" s="13" t="n"/>
@@ -1161,7 +1266,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G24" s="13" t="n"/>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="H24" s="13" t="n"/>
       <c r="I24" s="13" t="n"/>
       <c r="J24" s="13" t="n"/>
@@ -1189,7 +1298,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G25" s="13" t="n"/>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="H25" s="13" t="n"/>
       <c r="I25" s="13" t="n"/>
       <c r="J25" s="13" t="n"/>
@@ -1213,7 +1326,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G26" s="13" t="n"/>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H26" s="13" t="n"/>
       <c r="I26" s="13" t="n"/>
       <c r="J26" s="13" t="n"/>
@@ -1237,7 +1354,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G27" s="13" t="n"/>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H27" s="13" t="n"/>
       <c r="I27" s="13" t="n"/>
       <c r="J27" s="13" t="n"/>
@@ -1261,7 +1382,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G28" s="13" t="n"/>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H28" s="13" t="n"/>
       <c r="I28" s="13" t="n"/>
       <c r="J28" s="13" t="n"/>
@@ -1301,7 +1426,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G30" s="13" t="n"/>
+      <c r="G30" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H30" s="13" t="n"/>
       <c r="I30" s="13" t="n"/>
       <c r="J30" s="13" t="n"/>
@@ -1325,7 +1454,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G31" s="13" t="n"/>
+      <c r="G31" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H31" s="13" t="n"/>
       <c r="I31" s="13" t="n"/>
       <c r="J31" s="13" t="n"/>
@@ -1353,7 +1486,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G32" s="13" t="n"/>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H32" s="13" t="n"/>
       <c r="I32" s="13" t="n"/>
       <c r="J32" s="13" t="n"/>
@@ -1377,7 +1514,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G33" s="13" t="n"/>
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H33" s="13" t="n"/>
       <c r="I33" s="13" t="n"/>
       <c r="J33" s="13" t="n"/>
@@ -1401,7 +1542,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G34" s="13" t="n"/>
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H34" s="13" t="n"/>
       <c r="I34" s="13" t="n"/>
       <c r="J34" s="13" t="n"/>
@@ -1425,7 +1570,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G35" s="13" t="n"/>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H35" s="13" t="n"/>
       <c r="I35" s="13" t="n"/>
       <c r="J35" s="13" t="n"/>
@@ -1449,7 +1598,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G36" s="13" t="n"/>
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H36" s="13" t="n"/>
       <c r="I36" s="13" t="n"/>
       <c r="J36" s="13" t="n"/>
@@ -1473,7 +1626,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G37" s="13" t="n"/>
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H37" s="13" t="n"/>
       <c r="I37" s="13" t="n"/>
       <c r="J37" s="13" t="n"/>
@@ -1501,7 +1658,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G38" s="13" t="n"/>
+      <c r="G38" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H38" s="13" t="n"/>
       <c r="I38" s="13" t="n"/>
       <c r="J38" s="13" t="n"/>
@@ -1525,7 +1686,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G39" s="13" t="n"/>
+      <c r="G39" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H39" s="13" t="n"/>
       <c r="I39" s="13" t="n"/>
       <c r="J39" s="13" t="n"/>
@@ -1549,7 +1714,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G40" s="13" t="n"/>
+      <c r="G40" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H40" s="13" t="n"/>
       <c r="I40" s="13" t="n"/>
       <c r="J40" s="13" t="n"/>
@@ -1573,7 +1742,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G41" s="13" t="n"/>
+      <c r="G41" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H41" s="13" t="n"/>
       <c r="I41" s="13" t="n"/>
       <c r="J41" s="13" t="n"/>
@@ -1597,7 +1770,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G42" s="13" t="n"/>
+      <c r="G42" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H42" s="13" t="n"/>
       <c r="I42" s="13" t="n"/>
       <c r="J42" s="13" t="n"/>
@@ -1621,7 +1798,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G43" s="13" t="n"/>
+      <c r="G43" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H43" s="13" t="n"/>
       <c r="I43" s="13" t="n"/>
       <c r="J43" s="13" t="n"/>
@@ -1661,7 +1842,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G45" s="13" t="n"/>
+      <c r="G45" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H45" s="13" t="n"/>
       <c r="I45" s="13" t="n"/>
       <c r="J45" s="13" t="n"/>
@@ -1685,7 +1870,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G46" s="13" t="n"/>
+      <c r="G46" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H46" s="13" t="n"/>
       <c r="I46" s="13" t="n"/>
       <c r="J46" s="13" t="n"/>
@@ -1709,7 +1898,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G47" s="13" t="n"/>
+      <c r="G47" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H47" s="13" t="n"/>
       <c r="I47" s="13" t="n"/>
       <c r="J47" s="13" t="n"/>
@@ -1737,7 +1930,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G48" s="13" t="n"/>
+      <c r="G48" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H48" s="13" t="n"/>
       <c r="I48" s="13" t="n"/>
       <c r="J48" s="13" t="n"/>
@@ -1761,7 +1958,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G49" s="13" t="n"/>
+      <c r="G49" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H49" s="13" t="n"/>
       <c r="I49" s="13" t="n"/>
       <c r="J49" s="13" t="n"/>
@@ -1785,7 +1986,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G50" s="13" t="n"/>
+      <c r="G50" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H50" s="13" t="n"/>
       <c r="I50" s="13" t="n"/>
       <c r="J50" s="13" t="n"/>
@@ -1809,7 +2014,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G51" s="13" t="n"/>
+      <c r="G51" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H51" s="13" t="n"/>
       <c r="I51" s="13" t="n"/>
       <c r="J51" s="13" t="n"/>
@@ -1833,7 +2042,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G52" s="13" t="n"/>
+      <c r="G52" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H52" s="13" t="n"/>
       <c r="I52" s="13" t="n"/>
       <c r="J52" s="13" t="n"/>
@@ -1857,7 +2070,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G53" s="13" t="n"/>
+      <c r="G53" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H53" s="13" t="n"/>
       <c r="I53" s="13" t="n"/>
       <c r="J53" s="13" t="n"/>
@@ -1885,7 +2102,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G54" s="13" t="n"/>
+      <c r="G54" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H54" s="13" t="n"/>
       <c r="I54" s="13" t="n"/>
       <c r="J54" s="13" t="n"/>
@@ -1909,7 +2130,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G55" s="13" t="n"/>
+      <c r="G55" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H55" s="13" t="n"/>
       <c r="I55" s="13" t="n"/>
       <c r="J55" s="13" t="n"/>
@@ -1933,7 +2158,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G56" s="13" t="n"/>
+      <c r="G56" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H56" s="13" t="n"/>
       <c r="I56" s="13" t="n"/>
       <c r="J56" s="13" t="n"/>
@@ -1961,7 +2190,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G57" s="13" t="n"/>
+      <c r="G57" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H57" s="13" t="n"/>
       <c r="I57" s="13" t="n"/>
       <c r="J57" s="13" t="n"/>
@@ -1985,7 +2218,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G58" s="13" t="n"/>
+      <c r="G58" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H58" s="13" t="n"/>
       <c r="I58" s="13" t="n"/>
       <c r="J58" s="13" t="n"/>
@@ -2009,7 +2246,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G59" s="13" t="n"/>
+      <c r="G59" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H59" s="13" t="n"/>
       <c r="I59" s="13" t="n"/>
       <c r="J59" s="13" t="n"/>
@@ -2033,7 +2274,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G60" s="13" t="n"/>
+      <c r="G60" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H60" s="13" t="n"/>
       <c r="I60" s="13" t="n"/>
       <c r="J60" s="13" t="n"/>
@@ -2057,7 +2302,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G61" s="13" t="n"/>
+      <c r="G61" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H61" s="13" t="n"/>
       <c r="I61" s="13" t="n"/>
       <c r="J61" s="13" t="n"/>
@@ -2081,7 +2330,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G62" s="13" t="n"/>
+      <c r="G62" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H62" s="13" t="n"/>
       <c r="I62" s="13" t="n"/>
       <c r="J62" s="13" t="n"/>
@@ -2105,7 +2358,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G63" s="13" t="n"/>
+      <c r="G63" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H63" s="13" t="n"/>
       <c r="I63" s="13" t="n"/>
       <c r="J63" s="13" t="n"/>
@@ -2133,7 +2390,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G64" s="13" t="n"/>
+      <c r="G64" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H64" s="13" t="n"/>
       <c r="I64" s="13" t="n"/>
       <c r="J64" s="13" t="n"/>
@@ -2173,7 +2434,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G66" s="13" t="n"/>
+      <c r="G66" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H66" s="13" t="n"/>
       <c r="I66" s="13" t="n"/>
       <c r="J66" s="13" t="n"/>
@@ -2197,7 +2462,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G67" s="13" t="n"/>
+      <c r="G67" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H67" s="13" t="n"/>
       <c r="I67" s="13" t="n"/>
       <c r="J67" s="13" t="n"/>
@@ -2221,7 +2490,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G68" s="13" t="n"/>
+      <c r="G68" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H68" s="13" t="n"/>
       <c r="I68" s="13" t="n"/>
       <c r="J68" s="13" t="n"/>
@@ -2245,7 +2518,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G69" s="13" t="n"/>
+      <c r="G69" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H69" s="13" t="n"/>
       <c r="I69" s="13" t="n"/>
       <c r="J69" s="13" t="n"/>
@@ -2269,7 +2546,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G70" s="13" t="n"/>
+      <c r="G70" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H70" s="13" t="n"/>
       <c r="I70" s="13" t="n"/>
       <c r="J70" s="13" t="n"/>
@@ -2293,7 +2574,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G71" s="13" t="n"/>
+      <c r="G71" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H71" s="13" t="n"/>
       <c r="I71" s="13" t="n"/>
       <c r="J71" s="13" t="n"/>
@@ -2317,7 +2602,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G72" s="13" t="n"/>
+      <c r="G72" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H72" s="13" t="n"/>
       <c r="I72" s="13" t="n"/>
       <c r="J72" s="13" t="n"/>
@@ -2341,7 +2630,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G73" s="13" t="n"/>
+      <c r="G73" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H73" s="13" t="n"/>
       <c r="I73" s="13" t="n"/>
       <c r="J73" s="13" t="n"/>
@@ -2365,7 +2658,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G74" s="13" t="n"/>
+      <c r="G74" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H74" s="13" t="n"/>
       <c r="I74" s="13" t="n"/>
       <c r="J74" s="13" t="n"/>
@@ -2389,7 +2686,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G75" s="13" t="n"/>
+      <c r="G75" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H75" s="13" t="n"/>
       <c r="I75" s="13" t="n"/>
       <c r="J75" s="13" t="n"/>
@@ -2413,7 +2714,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G76" s="13" t="n"/>
+      <c r="G76" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="H76" s="13" t="n"/>
       <c r="I76" s="13" t="n"/>
       <c r="J76" s="13" t="n"/>
@@ -2437,7 +2742,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G77" s="13" t="n"/>
+      <c r="G77" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H77" s="13" t="n"/>
       <c r="I77" s="13" t="n"/>
       <c r="J77" s="13" t="n"/>
@@ -2465,7 +2774,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G78" s="13" t="n"/>
+      <c r="G78" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H78" s="13" t="n"/>
       <c r="I78" s="13" t="n"/>
       <c r="J78" s="13" t="n"/>
@@ -2489,7 +2802,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G79" s="13" t="n"/>
+      <c r="G79" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H79" s="13" t="n"/>
       <c r="I79" s="13" t="n"/>
       <c r="J79" s="13" t="n"/>
@@ -2513,7 +2830,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G80" s="13" t="n"/>
+      <c r="G80" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H80" s="13" t="n"/>
       <c r="I80" s="13" t="n"/>
       <c r="J80" s="13" t="n"/>
@@ -2537,7 +2858,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G81" s="13" t="n"/>
+      <c r="G81" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H81" s="13" t="n"/>
       <c r="I81" s="13" t="n"/>
       <c r="J81" s="13" t="n"/>
@@ -2561,7 +2886,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G82" s="13" t="n"/>
+      <c r="G82" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H82" s="13" t="n"/>
       <c r="I82" s="13" t="n"/>
       <c r="J82" s="13" t="n"/>
@@ -2605,7 +2934,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G84" s="13" t="n"/>
+      <c r="G84" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H84" s="13" t="n"/>
       <c r="I84" s="13" t="n"/>
       <c r="J84" s="13" t="n"/>
@@ -2629,7 +2962,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G85" s="13" t="n"/>
+      <c r="G85" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H85" s="13" t="n"/>
       <c r="I85" s="13" t="n"/>
       <c r="J85" s="13" t="n"/>
@@ -2653,7 +2990,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G86" s="13" t="n"/>
+      <c r="G86" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H86" s="13" t="n"/>
       <c r="I86" s="13" t="n"/>
       <c r="J86" s="13" t="n"/>
@@ -2677,7 +3018,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G87" s="13" t="n"/>
+      <c r="G87" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H87" s="13" t="n"/>
       <c r="I87" s="13" t="n"/>
       <c r="J87" s="13" t="n"/>
@@ -2701,7 +3046,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G88" s="13" t="n"/>
+      <c r="G88" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="H88" s="13" t="n"/>
       <c r="I88" s="13" t="n"/>
       <c r="J88" s="13" t="n"/>
@@ -2745,7 +3094,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G90" s="13" t="n"/>
+      <c r="G90" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H90" s="13" t="n"/>
       <c r="I90" s="13" t="n"/>
       <c r="J90" s="13" t="n"/>
@@ -2769,7 +3122,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G91" s="13" t="n"/>
+      <c r="G91" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="H91" s="13" t="n"/>
       <c r="I91" s="13" t="n"/>
       <c r="J91" s="13" t="n"/>
@@ -2793,7 +3150,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="G92" s="13" t="n"/>
+      <c r="G92" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="H92" s="13" t="n"/>
       <c r="I92" s="13" t="n"/>
       <c r="J92" s="13" t="n"/>
@@ -2817,7 +3178,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G93" s="13" t="n"/>
+      <c r="G93" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="H93" s="13" t="n"/>
       <c r="I93" s="13" t="n"/>
       <c r="J93" s="13" t="n"/>
@@ -3212,37 +3577,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H25"/>
+  <dimension ref="B2:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="78" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="86" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Rep 2 Review</t>
+          <t>Findings Log</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="32" t="inlineStr">
-        <is>
-          <t>Scored 72 / 78. Up from 57 / 78 on rep 1.</t>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Carried across reps. A finding stays open until the rebuild produces it correctly without prompting.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Every structural gap from rep 1 closed except one. What follows is what is left, ranked.</t>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Rep 1: 57/78   Rep 2: 72/78   Rep 3: 71/78 in 44 minutes</t>
         </is>
       </c>
     </row>
@@ -3254,447 +3617,399 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Since</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
           <t>Finding</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Why it matters</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="58" customHeight="1">
+    </row>
+    <row r="8" ht="46" customHeight="1">
       <c r="B8" s="17" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C8" s="33" t="inlineStr">
-        <is>
-          <t>BUG</t>
-        </is>
-      </c>
-      <c r="D8" s="17" t="inlineStr">
-        <is>
-          <t>Revolver repayment has no cap</t>
-        </is>
-      </c>
-      <c r="E8" s="30">
-        <f>IF(D181&gt;D180,(D181-D180),0) repays the full excess over minimum cash, even when you owe less than that. The revolver goes negative. Your test numbers (cash 70, min 50, owed 20) are the one case where excess exactly equals the balance, so it could not show. Fix: =MIN(beginning balance, MAX(0, cash - minimum)).</f>
-        <v/>
-      </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>Drill 3 on the drills page. This is precisely the cap it exists to teach.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="58" customHeight="1">
+      <c r="C8" s="43" t="inlineStr">
+        <is>
+          <t>Rep 2</t>
+        </is>
+      </c>
+      <c r="D8" s="44" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>Income taxes payable absent from the balance sheet</t>
+        </is>
+      </c>
+      <c r="F8" s="30" t="inlineStr">
+        <is>
+          <t>Now at B70 in current liabilities. This was your only repeat miss and it is closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C9" s="35" t="inlineStr">
-        <is>
-          <t>WIRING</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="inlineStr">
-        <is>
-          <t>Revolver reads final cash, not cash before the revolver</t>
-        </is>
-      </c>
-      <c r="E9" s="30" t="inlineStr">
-        <is>
-          <t>D181 links to the balance sheet cash line. That line is the OUTPUT of the sweep, so once you add numbers this becomes circular in the wrong way. It must reference cash before any revolver activity: opening cash + CFO + CFI + financing excluding the revolver.</t>
-        </is>
-      </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>Bites on Day 6 when the model first closes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="58" customHeight="1">
+      <c r="C9" s="43" t="inlineStr">
+        <is>
+          <t>Rep 2</t>
+        </is>
+      </c>
+      <c r="D9" s="44" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>No effective tax rate assumption</t>
+        </is>
+      </c>
+      <c r="F9" s="30" t="inlineStr">
+        <is>
+          <t>B16 now reads 'Effective Tax Rate'. The rep 2 row said 'Effective interest rate' - it was the typing slip it looked like.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
       <c r="B10" s="17" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C10" s="33" t="inlineStr">
-        <is>
-          <t>MISS</t>
-        </is>
-      </c>
-      <c r="D10" s="17" t="inlineStr">
-        <is>
-          <t>Income taxes payable is still absent from the balance sheet</t>
-        </is>
-      </c>
-      <c r="E10" s="30" t="inlineStr">
-        <is>
-          <t>You have the days assumption (B14), the working capital schedule line (B128) and the cash flow line (B102) - but no balance in current liabilities. Same miss as rep 1. A line that flows through the CFS must have a home on the BS.</t>
-        </is>
-      </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>This is your one repeat error. Put it on the next rep's checklist first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="58" customHeight="1">
+      <c r="C10" s="43" t="inlineStr">
+        <is>
+          <t>Rep 2</t>
+        </is>
+      </c>
+      <c r="D10" s="44" t="inlineStr">
+        <is>
+          <t>IMPROVED</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>Debt schedule was too thin</t>
+        </is>
+      </c>
+      <c r="F10" s="30" t="inlineStr">
+        <is>
+          <t>Now beginning / repayment / interest expense / ending. Still no draws-or-issuance line, so the roll-forward can only shrink: beginning - repayment = ending. Add the additions row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
       <c r="B11" s="17" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C11" s="35" t="inlineStr">
-        <is>
-          <t>WRONG PLACE</t>
-        </is>
-      </c>
-      <c r="D11" s="17" t="inlineStr">
-        <is>
-          <t>'Dividends' sits as a line inside shareholders' equity</t>
-        </is>
-      </c>
-      <c r="E11" s="30" t="inlineStr">
-        <is>
-          <t>B82. Dividends are a flow, not a balance. They belong on the income statement, in financing on the cash flow statement, and as a deduction inside the equity roll-forward - not as a standing balance sheet row.</t>
-        </is>
-      </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>Delete the row; the equity schedule already handles it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="58" customHeight="1">
+      <c r="C11" s="43" t="inlineStr">
+        <is>
+          <t>Rep 3</t>
+        </is>
+      </c>
+      <c r="D11" s="33" t="inlineStr">
+        <is>
+          <t>REGRESSED</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>Revolver schedule is now an empty header</t>
+        </is>
+      </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>Rows 175-177 carry the title, the units note and the date row - and nothing else. Rep 2 had a working block with live draw and repayment formulas. It was not rebuilt this time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
       <c r="B12" s="17" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C12" s="35" t="inlineStr">
-        <is>
-          <t>SLIP</t>
-        </is>
-      </c>
-      <c r="D12" s="17" t="inlineStr">
-        <is>
-          <t>No effective tax rate assumption</t>
-        </is>
-      </c>
-      <c r="E12" s="30" t="inlineStr">
-        <is>
-          <t>B15 reads 'Effective interest rate', sitting directly above three other interest rate lines. You have a Taxes line on the income statement and an income-tax-payable days driver, so the tax rate is what that row was meant to be.</t>
-        </is>
-      </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>Almost certainly a typing slip rather than a recall failure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="58" customHeight="1">
+      <c r="C12" s="43" t="inlineStr">
+        <is>
+          <t>Rep 3</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>REGRESSED</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>Revolver rate and minimum cash assumptions dropped</t>
+        </is>
+      </c>
+      <c r="F12" s="30" t="inlineStr">
+        <is>
+          <t>Both were present in rep 2 and are gone from the assumptions block. Without a minimum cash balance the sweep has nothing to solve against.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
       <c r="B13" s="17" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C13" s="35" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D13" s="17" t="inlineStr">
+      <c r="C13" s="43" t="inlineStr">
+        <is>
+          <t>Rep 2</t>
+        </is>
+      </c>
+      <c r="D13" s="45" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>'Dividends' still sits as a row inside shareholders' equity</t>
+        </is>
+      </c>
+      <c r="F13" s="30" t="inlineStr">
+        <is>
+          <t>B81. Flagged last rep, unchanged. Dividends are a flow - income statement, financing on the CFS, and a deduction inside the equity roll-forward. Not a balance sheet row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C14" s="43" t="inlineStr">
+        <is>
+          <t>Rep 2</t>
+        </is>
+      </c>
+      <c r="D14" s="45" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
         <is>
           <t>No revolver line in cash flow financing</t>
         </is>
       </c>
-      <c r="E13" s="30" t="inlineStr">
-        <is>
-          <t>The financing section has debt, equity and dividends. The revolver draw and repayment need their own line there so the sweep actually moves cash.</t>
-        </is>
-      </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>Minor - you built the schedule, it just is not wired to the CFS yet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="58" customHeight="1">
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C14" s="35" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D14" s="17" t="inlineStr">
-        <is>
-          <t>No mandatory debt amortisation</t>
-        </is>
-      </c>
-      <c r="E14" s="30" t="inlineStr">
-        <is>
-          <t>The debt schedule is beginning + issuance = ending. A real one also has the scheduled repayment as its own line.</t>
-        </is>
-      </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>Add on Day 8.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="58" customHeight="1">
+      <c r="F14" s="30" t="inlineStr">
+        <is>
+          <t>Financing still has debt, equity and dividends only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="46" customHeight="1">
       <c r="B15" s="17" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="C15" s="35" t="inlineStr">
-        <is>
-          <t>STRUCTURE</t>
-        </is>
-      </c>
-      <c r="D15" s="17" t="inlineStr">
+      <c r="C15" s="43" t="inlineStr">
+        <is>
+          <t>Rep 2</t>
+        </is>
+      </c>
+      <c r="D15" s="45" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
         <is>
           <t>No colour convention anywhere</t>
         </is>
       </c>
-      <c r="E15" s="30" t="inlineStr">
-        <is>
-          <t>Every cell in the file uses the default theme font. Blue for hardcoded inputs, black for formulas, green for cross-sheet links. Start this now, while the model is small enough that it costs nothing.</t>
-        </is>
-      </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>Also: mark which periods are actual and which are projected.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="58" customHeight="1">
+      <c r="F15" s="30" t="inlineStr">
+        <is>
+          <t>All 203 populated cells still use the default theme font. Blue inputs, black formulas, green cross-sheet links.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="46" customHeight="1">
       <c r="B16" s="17" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="C16" s="35" t="inlineStr">
-        <is>
-          <t>NIT</t>
-        </is>
-      </c>
-      <c r="D16" s="17" t="inlineStr">
-        <is>
-          <t>Cash from Operations header sits below net income</t>
-        </is>
-      </c>
-      <c r="E16" s="30" t="inlineStr">
-        <is>
-          <t>B98 is a section header but it appears after net income and depreciation. Move it above B95 so the section reads top-down.</t>
-        </is>
-      </c>
-      <c r="F16" s="34" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>WHY THE REVOLVER FORMULA FAILS</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="36" t="inlineStr">
-        <is>
-          <t>Edit the blue cells - the two columns disagree whenever excess cash exceeds what you owe.</t>
+      <c r="C16" s="43" t="inlineStr">
+        <is>
+          <t>Rep 2</t>
+        </is>
+      </c>
+      <c r="D16" s="45" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>'Cash from Operations' header sits below net income</t>
+        </is>
+      </c>
+      <c r="F16" s="30" t="inlineStr">
+        <is>
+          <t>B97, after net income and depreciation. Move it above so the section reads top-down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="46" customHeight="1">
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C17" s="43" t="inlineStr">
+        <is>
+          <t>Rep 3</t>
+        </is>
+      </c>
+      <c r="D17" s="45" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>No actual vs. projected markers on the periods</t>
+        </is>
+      </c>
+      <c r="F17" s="30" t="inlineStr">
+        <is>
+          <t>Eight periods now run 2022 to 2029, but nothing says where history stops and the forecast starts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="46" customHeight="1">
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C18" s="43" t="inlineStr">
+        <is>
+          <t>Rep 3</t>
+        </is>
+      </c>
+      <c r="D18" s="35" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>Day 2's layer was not attempted</t>
+        </is>
+      </c>
+      <c r="F18" s="30" t="inlineStr">
+        <is>
+          <t>The ladder's Day 2 is periods PLUS assumption values. There is not a single number in the file - this was another skeleton rep. Not wrong, but the layer is still outstanding.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="37" t="inlineStr">
-        <is>
-          <t>Beginning</t>
-        </is>
-      </c>
-      <c r="C20" s="37" t="inlineStr">
-        <is>
-          <t>Cash</t>
-        </is>
-      </c>
-      <c r="D20" s="37" t="inlineStr">
-        <is>
-          <t>Min cash</t>
-        </is>
-      </c>
-      <c r="E20" s="37" t="inlineStr">
-        <is>
-          <t>Yours: repay</t>
-        </is>
-      </c>
-      <c r="F20" s="37" t="inlineStr">
-        <is>
-          <t>Yours: ending</t>
-        </is>
-      </c>
-      <c r="G20" s="37" t="inlineStr">
-        <is>
-          <t>Correct: repay</t>
-        </is>
-      </c>
-      <c r="H20" s="37" t="inlineStr">
-        <is>
-          <t>Correct: ending</t>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>NEXT REP - fix list, in order</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="38" t="n">
-        <v>20</v>
-      </c>
-      <c r="C21" s="38" t="n">
-        <v>70</v>
-      </c>
-      <c r="D21" s="38" t="n">
-        <v>50</v>
-      </c>
-      <c r="E21" s="39">
-        <f>IF(C21&gt;D21,(C21-D21),0)</f>
-        <v/>
-      </c>
-      <c r="F21" s="40">
-        <f>B21-E21</f>
-        <v/>
-      </c>
-      <c r="G21" s="39">
-        <f>MIN(B21,MAX(0,C21-D21))</f>
-        <v/>
-      </c>
-      <c r="H21" s="41">
-        <f>B21-G21</f>
-        <v/>
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C21" s="25" t="inlineStr">
+        <is>
+          <t>Rebuild the revolver block and put its two assumptions back (findings 4 and 5).</t>
+        </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="38" t="n">
-        <v>20</v>
-      </c>
-      <c r="C22" s="38" t="n">
-        <v>100</v>
-      </c>
-      <c r="D22" s="38" t="n">
-        <v>50</v>
-      </c>
-      <c r="E22" s="39">
-        <f>IF(C22&gt;D22,(C22-D22),0)</f>
-        <v/>
-      </c>
-      <c r="F22" s="40">
-        <f>B22-E22</f>
-        <v/>
-      </c>
-      <c r="G22" s="39">
-        <f>MIN(B22,MAX(0,C22-D22))</f>
-        <v/>
-      </c>
-      <c r="H22" s="41">
-        <f>B22-G22</f>
-        <v/>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C22" s="25" t="inlineStr">
+        <is>
+          <t>Delete the Dividends row from shareholders' equity (finding 6).</t>
+        </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="C23" s="38" t="n">
-        <v>120</v>
-      </c>
-      <c r="D23" s="38" t="n">
-        <v>50</v>
-      </c>
-      <c r="E23" s="39">
-        <f>IF(C23&gt;D23,(C23-D23),0)</f>
-        <v/>
-      </c>
-      <c r="F23" s="40">
-        <f>B23-E23</f>
-        <v/>
-      </c>
-      <c r="G23" s="39">
-        <f>MIN(B23,MAX(0,C23-D23))</f>
-        <v/>
-      </c>
-      <c r="H23" s="41">
-        <f>B23-G23</f>
-        <v/>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C23" s="25" t="inlineStr">
+        <is>
+          <t>Add a revolver line to cash flow financing (finding 7).</t>
+        </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="38" t="n">
-        <v>10</v>
-      </c>
-      <c r="C24" s="38" t="n">
-        <v>200</v>
-      </c>
-      <c r="D24" s="38" t="n">
-        <v>50</v>
-      </c>
-      <c r="E24" s="39">
-        <f>IF(C24&gt;D24,(C24-D24),0)</f>
-        <v/>
-      </c>
-      <c r="F24" s="40">
-        <f>B24-E24</f>
-        <v/>
-      </c>
-      <c r="G24" s="39">
-        <f>MIN(B24,MAX(0,C24-D24))</f>
-        <v/>
-      </c>
-      <c r="H24" s="41">
-        <f>B24-G24</f>
-        <v/>
+      <c r="B24" s="23" t="inlineStr">
+        <is>
+          <t>4.</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="inlineStr">
+        <is>
+          <t>Add the draws row to the debt schedule (finding 3).</t>
+        </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="38" t="n">
-        <v>20</v>
-      </c>
-      <c r="C25" s="38" t="n">
-        <v>30</v>
-      </c>
-      <c r="D25" s="38" t="n">
-        <v>50</v>
-      </c>
-      <c r="E25" s="39">
-        <f>IF(C25&gt;D25,(C25-D25),0)</f>
-        <v/>
-      </c>
-      <c r="F25" s="40">
-        <f>B25-E25</f>
-        <v/>
-      </c>
-      <c r="G25" s="39">
-        <f>MIN(B25,MAX(0,C25-D25))</f>
-        <v/>
-      </c>
-      <c r="H25" s="41">
-        <f>B25-G25</f>
-        <v/>
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>5.</t>
+        </is>
+      </c>
+      <c r="C25" s="25" t="inlineStr">
+        <is>
+          <t>Colour every cell as you type it - blue, black, green (finding 8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>6.</t>
+        </is>
+      </c>
+      <c r="C26" s="25" t="inlineStr">
+        <is>
+          <t>Then, and only then, enter assumption values. That is the Day 2 layer.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3956,15 +4271,15 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1">
+    <row r="9" ht="44" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="C9" s="29" t="inlineStr">
-        <is>
-          <t>DONE</t>
+      <c r="C9" s="46" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="D9" s="17" t="inlineStr">
@@ -3974,7 +4289,7 @@
       </c>
       <c r="E9" s="30" t="inlineStr">
         <is>
-          <t>Skeleton rebuilt at 72/78 with all four schedules and a working revolver block. Periods, subtotals and balance check added. Next: fix the six findings, then add assumption values.</t>
+          <t>Skeleton rebuilt in 44 min at 71/78. Balance sheet perfect, tax rate and taxes-payable fixed. Revolver block and its assumptions regressed. Assumption VALUES still outstanding - repeat Day 2.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Score rep 4, a seven-page paper skeleton
Scores 70/74 on the content blocks, tying the best result so far, with
the cash flow statement complete for the first time at 17/17. Seven
findings close this rep, including two that had been open since rep 2.

Adds a medium row and a content-only percentage that excludes the four
Structure items, since a paper rep cannot demonstrate period headers or
a colour convention and the raw score would understate it.

Records the recurring pattern explicitly: each rep closes the flagged
findings and drops something previously solid, which points at a closing
verification sweep rather than harder recall.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UX5HPwj2AEakAb4LMEQ7Bv
</commit_message>
<xml_diff>
--- a/learning/model-practice/Day_2_scorecard_and_ladder.xlsx
+++ b/learning/model-practice/Day_2_scorecard_and_ladder.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="25">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -167,8 +167,32 @@
       <color rgb="FFB26B00"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1546C9"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1546C9"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFC00000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -200,6 +224,11 @@
         <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF0F0F0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -227,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -309,6 +338,22 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -674,7 +719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:K104"/>
+  <dimension ref="B2:K105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -711,6 +756,38 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D5" s="36" t="inlineStr">
+        <is>
+          <t>Paper reps cannot show the Structure block - score those on the 74 content items</t>
+        </is>
+      </c>
+      <c r="E5" s="47" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="F5" s="47" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="G5" s="47" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="H5" s="48" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -891,7 +968,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H11" s="13" t="n"/>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I11" s="13" t="n"/>
       <c r="J11" s="13" t="n"/>
       <c r="K11" s="13" t="n"/>
@@ -919,7 +1000,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H12" s="13" t="n"/>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I12" s="13" t="n"/>
       <c r="J12" s="13" t="n"/>
       <c r="K12" s="13" t="n"/>
@@ -947,7 +1032,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H13" s="13" t="n"/>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I13" s="13" t="n"/>
       <c r="J13" s="13" t="n"/>
       <c r="K13" s="13" t="n"/>
@@ -975,7 +1064,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H14" s="13" t="n"/>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I14" s="13" t="n"/>
       <c r="J14" s="13" t="n"/>
       <c r="K14" s="13" t="n"/>
@@ -1007,7 +1100,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H15" s="13" t="n"/>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I15" s="13" t="n"/>
       <c r="J15" s="13" t="n"/>
       <c r="K15" s="13" t="n"/>
@@ -1035,7 +1132,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H16" s="13" t="n"/>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I16" s="13" t="n"/>
       <c r="J16" s="13" t="n"/>
       <c r="K16" s="13" t="n"/>
@@ -1063,7 +1164,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H17" s="13" t="n"/>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I17" s="13" t="n"/>
       <c r="J17" s="13" t="n"/>
       <c r="K17" s="13" t="n"/>
@@ -1091,7 +1196,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H18" s="13" t="n"/>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I18" s="13" t="n"/>
       <c r="J18" s="13" t="n"/>
       <c r="K18" s="13" t="n"/>
@@ -1119,7 +1228,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H19" s="13" t="n"/>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I19" s="13" t="n"/>
       <c r="J19" s="13" t="n"/>
       <c r="K19" s="13" t="n"/>
@@ -1151,7 +1264,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H20" s="13" t="n"/>
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I20" s="13" t="n"/>
       <c r="J20" s="13" t="n"/>
       <c r="K20" s="13" t="n"/>
@@ -1179,7 +1296,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H21" s="13" t="n"/>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I21" s="13" t="n"/>
       <c r="J21" s="13" t="n"/>
       <c r="K21" s="13" t="n"/>
@@ -1207,7 +1328,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H22" s="13" t="n"/>
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I22" s="13" t="n"/>
       <c r="J22" s="13" t="n"/>
       <c r="K22" s="13" t="n"/>
@@ -1239,7 +1364,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H23" s="13" t="n"/>
+      <c r="H23" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I23" s="13" t="n"/>
       <c r="J23" s="13" t="n"/>
       <c r="K23" s="13" t="n"/>
@@ -1271,7 +1400,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H24" s="13" t="n"/>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I24" s="13" t="n"/>
       <c r="J24" s="13" t="n"/>
       <c r="K24" s="13" t="n"/>
@@ -1303,7 +1436,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H25" s="13" t="n"/>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I25" s="13" t="n"/>
       <c r="J25" s="13" t="n"/>
       <c r="K25" s="13" t="n"/>
@@ -1331,7 +1468,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H26" s="13" t="n"/>
+      <c r="H26" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I26" s="13" t="n"/>
       <c r="J26" s="13" t="n"/>
       <c r="K26" s="13" t="n"/>
@@ -1359,7 +1500,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H27" s="13" t="n"/>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I27" s="13" t="n"/>
       <c r="J27" s="13" t="n"/>
       <c r="K27" s="13" t="n"/>
@@ -1387,7 +1532,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H28" s="13" t="n"/>
+      <c r="H28" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I28" s="13" t="n"/>
       <c r="J28" s="13" t="n"/>
       <c r="K28" s="13" t="n"/>
@@ -1431,7 +1580,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H30" s="13" t="n"/>
+      <c r="H30" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I30" s="13" t="n"/>
       <c r="J30" s="13" t="n"/>
       <c r="K30" s="13" t="n"/>
@@ -1459,7 +1612,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H31" s="13" t="n"/>
+      <c r="H31" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I31" s="13" t="n"/>
       <c r="J31" s="13" t="n"/>
       <c r="K31" s="13" t="n"/>
@@ -1491,7 +1648,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H32" s="13" t="n"/>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I32" s="13" t="n"/>
       <c r="J32" s="13" t="n"/>
       <c r="K32" s="13" t="n"/>
@@ -1519,7 +1680,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H33" s="13" t="n"/>
+      <c r="H33" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I33" s="13" t="n"/>
       <c r="J33" s="13" t="n"/>
       <c r="K33" s="13" t="n"/>
@@ -1547,7 +1712,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H34" s="13" t="n"/>
+      <c r="H34" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I34" s="13" t="n"/>
       <c r="J34" s="13" t="n"/>
       <c r="K34" s="13" t="n"/>
@@ -1575,7 +1744,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H35" s="13" t="n"/>
+      <c r="H35" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I35" s="13" t="n"/>
       <c r="J35" s="13" t="n"/>
       <c r="K35" s="13" t="n"/>
@@ -1603,7 +1776,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H36" s="13" t="n"/>
+      <c r="H36" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I36" s="13" t="n"/>
       <c r="J36" s="13" t="n"/>
       <c r="K36" s="13" t="n"/>
@@ -1631,7 +1808,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H37" s="13" t="n"/>
+      <c r="H37" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I37" s="13" t="n"/>
       <c r="J37" s="13" t="n"/>
       <c r="K37" s="13" t="n"/>
@@ -1663,7 +1844,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H38" s="13" t="n"/>
+      <c r="H38" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I38" s="13" t="n"/>
       <c r="J38" s="13" t="n"/>
       <c r="K38" s="13" t="n"/>
@@ -1691,7 +1876,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H39" s="13" t="n"/>
+      <c r="H39" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I39" s="13" t="n"/>
       <c r="J39" s="13" t="n"/>
       <c r="K39" s="13" t="n"/>
@@ -1719,7 +1908,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H40" s="13" t="n"/>
+      <c r="H40" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I40" s="13" t="n"/>
       <c r="J40" s="13" t="n"/>
       <c r="K40" s="13" t="n"/>
@@ -1747,7 +1940,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H41" s="13" t="n"/>
+      <c r="H41" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I41" s="13" t="n"/>
       <c r="J41" s="13" t="n"/>
       <c r="K41" s="13" t="n"/>
@@ -1775,7 +1972,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H42" s="13" t="n"/>
+      <c r="H42" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I42" s="13" t="n"/>
       <c r="J42" s="13" t="n"/>
       <c r="K42" s="13" t="n"/>
@@ -1803,7 +2004,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H43" s="13" t="n"/>
+      <c r="H43" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I43" s="13" t="n"/>
       <c r="J43" s="13" t="n"/>
       <c r="K43" s="13" t="n"/>
@@ -1847,7 +2052,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H45" s="13" t="n"/>
+      <c r="H45" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I45" s="13" t="n"/>
       <c r="J45" s="13" t="n"/>
       <c r="K45" s="13" t="n"/>
@@ -1875,7 +2084,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H46" s="13" t="n"/>
+      <c r="H46" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I46" s="13" t="n"/>
       <c r="J46" s="13" t="n"/>
       <c r="K46" s="13" t="n"/>
@@ -1903,7 +2116,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H47" s="13" t="n"/>
+      <c r="H47" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I47" s="13" t="n"/>
       <c r="J47" s="13" t="n"/>
       <c r="K47" s="13" t="n"/>
@@ -1935,7 +2152,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H48" s="13" t="n"/>
+      <c r="H48" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I48" s="13" t="n"/>
       <c r="J48" s="13" t="n"/>
       <c r="K48" s="13" t="n"/>
@@ -1963,7 +2184,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H49" s="13" t="n"/>
+      <c r="H49" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I49" s="13" t="n"/>
       <c r="J49" s="13" t="n"/>
       <c r="K49" s="13" t="n"/>
@@ -1991,7 +2216,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H50" s="13" t="n"/>
+      <c r="H50" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I50" s="13" t="n"/>
       <c r="J50" s="13" t="n"/>
       <c r="K50" s="13" t="n"/>
@@ -2019,7 +2248,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H51" s="13" t="n"/>
+      <c r="H51" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I51" s="13" t="n"/>
       <c r="J51" s="13" t="n"/>
       <c r="K51" s="13" t="n"/>
@@ -2047,7 +2280,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H52" s="13" t="n"/>
+      <c r="H52" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I52" s="13" t="n"/>
       <c r="J52" s="13" t="n"/>
       <c r="K52" s="13" t="n"/>
@@ -2075,7 +2312,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H53" s="13" t="n"/>
+      <c r="H53" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I53" s="13" t="n"/>
       <c r="J53" s="13" t="n"/>
       <c r="K53" s="13" t="n"/>
@@ -2107,7 +2348,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H54" s="13" t="n"/>
+      <c r="H54" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I54" s="13" t="n"/>
       <c r="J54" s="13" t="n"/>
       <c r="K54" s="13" t="n"/>
@@ -2135,7 +2380,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H55" s="13" t="n"/>
+      <c r="H55" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I55" s="13" t="n"/>
       <c r="J55" s="13" t="n"/>
       <c r="K55" s="13" t="n"/>
@@ -2163,7 +2412,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H56" s="13" t="n"/>
+      <c r="H56" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I56" s="13" t="n"/>
       <c r="J56" s="13" t="n"/>
       <c r="K56" s="13" t="n"/>
@@ -2195,7 +2448,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H57" s="13" t="n"/>
+      <c r="H57" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I57" s="13" t="n"/>
       <c r="J57" s="13" t="n"/>
       <c r="K57" s="13" t="n"/>
@@ -2223,7 +2480,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H58" s="13" t="n"/>
+      <c r="H58" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I58" s="13" t="n"/>
       <c r="J58" s="13" t="n"/>
       <c r="K58" s="13" t="n"/>
@@ -2251,7 +2512,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H59" s="13" t="n"/>
+      <c r="H59" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I59" s="13" t="n"/>
       <c r="J59" s="13" t="n"/>
       <c r="K59" s="13" t="n"/>
@@ -2279,7 +2544,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H60" s="13" t="n"/>
+      <c r="H60" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I60" s="13" t="n"/>
       <c r="J60" s="13" t="n"/>
       <c r="K60" s="13" t="n"/>
@@ -2307,7 +2576,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H61" s="13" t="n"/>
+      <c r="H61" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I61" s="13" t="n"/>
       <c r="J61" s="13" t="n"/>
       <c r="K61" s="13" t="n"/>
@@ -2335,7 +2608,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H62" s="13" t="n"/>
+      <c r="H62" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I62" s="13" t="n"/>
       <c r="J62" s="13" t="n"/>
       <c r="K62" s="13" t="n"/>
@@ -2363,7 +2640,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H63" s="13" t="n"/>
+      <c r="H63" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I63" s="13" t="n"/>
       <c r="J63" s="13" t="n"/>
       <c r="K63" s="13" t="n"/>
@@ -2395,7 +2676,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H64" s="13" t="n"/>
+      <c r="H64" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I64" s="13" t="n"/>
       <c r="J64" s="13" t="n"/>
       <c r="K64" s="13" t="n"/>
@@ -2439,7 +2724,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H66" s="13" t="n"/>
+      <c r="H66" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I66" s="13" t="n"/>
       <c r="J66" s="13" t="n"/>
       <c r="K66" s="13" t="n"/>
@@ -2467,7 +2756,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H67" s="13" t="n"/>
+      <c r="H67" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I67" s="13" t="n"/>
       <c r="J67" s="13" t="n"/>
       <c r="K67" s="13" t="n"/>
@@ -2495,7 +2788,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H68" s="13" t="n"/>
+      <c r="H68" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I68" s="13" t="n"/>
       <c r="J68" s="13" t="n"/>
       <c r="K68" s="13" t="n"/>
@@ -2523,7 +2820,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H69" s="13" t="n"/>
+      <c r="H69" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I69" s="13" t="n"/>
       <c r="J69" s="13" t="n"/>
       <c r="K69" s="13" t="n"/>
@@ -2551,7 +2852,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H70" s="13" t="n"/>
+      <c r="H70" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I70" s="13" t="n"/>
       <c r="J70" s="13" t="n"/>
       <c r="K70" s="13" t="n"/>
@@ -2579,7 +2884,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H71" s="13" t="n"/>
+      <c r="H71" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I71" s="13" t="n"/>
       <c r="J71" s="13" t="n"/>
       <c r="K71" s="13" t="n"/>
@@ -2607,7 +2916,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H72" s="13" t="n"/>
+      <c r="H72" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I72" s="13" t="n"/>
       <c r="J72" s="13" t="n"/>
       <c r="K72" s="13" t="n"/>
@@ -2635,7 +2948,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H73" s="13" t="n"/>
+      <c r="H73" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I73" s="13" t="n"/>
       <c r="J73" s="13" t="n"/>
       <c r="K73" s="13" t="n"/>
@@ -2663,7 +2980,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H74" s="13" t="n"/>
+      <c r="H74" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I74" s="13" t="n"/>
       <c r="J74" s="13" t="n"/>
       <c r="K74" s="13" t="n"/>
@@ -2691,7 +3012,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H75" s="13" t="n"/>
+      <c r="H75" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I75" s="13" t="n"/>
       <c r="J75" s="13" t="n"/>
       <c r="K75" s="13" t="n"/>
@@ -2719,7 +3044,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H76" s="13" t="n"/>
+      <c r="H76" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I76" s="13" t="n"/>
       <c r="J76" s="13" t="n"/>
       <c r="K76" s="13" t="n"/>
@@ -2747,7 +3076,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H77" s="13" t="n"/>
+      <c r="H77" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I77" s="13" t="n"/>
       <c r="J77" s="13" t="n"/>
       <c r="K77" s="13" t="n"/>
@@ -2779,7 +3112,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H78" s="13" t="n"/>
+      <c r="H78" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I78" s="13" t="n"/>
       <c r="J78" s="13" t="n"/>
       <c r="K78" s="13" t="n"/>
@@ -2807,7 +3144,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H79" s="13" t="n"/>
+      <c r="H79" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I79" s="13" t="n"/>
       <c r="J79" s="13" t="n"/>
       <c r="K79" s="13" t="n"/>
@@ -2835,7 +3176,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H80" s="13" t="n"/>
+      <c r="H80" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I80" s="13" t="n"/>
       <c r="J80" s="13" t="n"/>
       <c r="K80" s="13" t="n"/>
@@ -2863,7 +3208,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H81" s="13" t="n"/>
+      <c r="H81" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I81" s="13" t="n"/>
       <c r="J81" s="13" t="n"/>
       <c r="K81" s="13" t="n"/>
@@ -2891,7 +3240,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H82" s="13" t="n"/>
+      <c r="H82" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I82" s="13" t="n"/>
       <c r="J82" s="13" t="n"/>
       <c r="K82" s="13" t="n"/>
@@ -2939,7 +3292,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H84" s="13" t="n"/>
+      <c r="H84" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I84" s="13" t="n"/>
       <c r="J84" s="13" t="n"/>
       <c r="K84" s="13" t="n"/>
@@ -2967,7 +3324,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H85" s="13" t="n"/>
+      <c r="H85" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I85" s="13" t="n"/>
       <c r="J85" s="13" t="n"/>
       <c r="K85" s="13" t="n"/>
@@ -2995,7 +3356,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H86" s="13" t="n"/>
+      <c r="H86" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I86" s="13" t="n"/>
       <c r="J86" s="13" t="n"/>
       <c r="K86" s="13" t="n"/>
@@ -3023,7 +3388,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H87" s="13" t="n"/>
+      <c r="H87" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I87" s="13" t="n"/>
       <c r="J87" s="13" t="n"/>
       <c r="K87" s="13" t="n"/>
@@ -3051,7 +3420,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H88" s="13" t="n"/>
+      <c r="H88" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I88" s="13" t="n"/>
       <c r="J88" s="13" t="n"/>
       <c r="K88" s="13" t="n"/>
@@ -3099,7 +3472,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H90" s="13" t="n"/>
+      <c r="H90" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I90" s="13" t="n"/>
       <c r="J90" s="13" t="n"/>
       <c r="K90" s="13" t="n"/>
@@ -3127,7 +3504,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H91" s="13" t="n"/>
+      <c r="H91" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I91" s="13" t="n"/>
       <c r="J91" s="13" t="n"/>
       <c r="K91" s="13" t="n"/>
@@ -3155,7 +3536,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="H92" s="13" t="n"/>
+      <c r="H92" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I92" s="13" t="n"/>
       <c r="J92" s="13" t="n"/>
       <c r="K92" s="13" t="n"/>
@@ -3183,7 +3568,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H93" s="13" t="n"/>
+      <c r="H93" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I93" s="13" t="n"/>
       <c r="J93" s="13" t="n"/>
       <c r="K93" s="13" t="n"/>
@@ -3558,6 +3947,51 @@
       </c>
       <c r="K104" s="21">
         <f>IF(COUNTA(K10:K93)=0,"",COUNTIF(K10:K93,"Y")/COUNTA(C10:C93))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>Content only</t>
+        </is>
+      </c>
+      <c r="C105" s="50" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="D105" s="36" t="inlineStr">
+        <is>
+          <t>Excludes the 4 Structure items so paper and Excel reps compare fairly</t>
+        </is>
+      </c>
+      <c r="E105" s="51">
+        <f>IF(COUNTA(E10:E93)=0,"",COUNTIF(E10:E89,"Y")/74)</f>
+        <v/>
+      </c>
+      <c r="F105" s="51">
+        <f>IF(COUNTA(F10:F93)=0,"",COUNTIF(F10:F89,"Y")/74)</f>
+        <v/>
+      </c>
+      <c r="G105" s="51">
+        <f>IF(COUNTA(G10:G93)=0,"",COUNTIF(G10:G89,"Y")/74)</f>
+        <v/>
+      </c>
+      <c r="H105" s="51">
+        <f>IF(COUNTA(H10:H93)=0,"",COUNTIF(H10:H89,"Y")/74)</f>
+        <v/>
+      </c>
+      <c r="I105" s="51">
+        <f>IF(COUNTA(I10:I93)=0,"",COUNTIF(I10:I89,"Y")/74)</f>
+        <v/>
+      </c>
+      <c r="J105" s="51">
+        <f>IF(COUNTA(J10:J93)=0,"",COUNTIF(J10:J89,"Y")/74)</f>
+        <v/>
+      </c>
+      <c r="K105" s="51">
+        <f>IF(COUNTA(K10:K93)=0,"",COUNTIF(K10:K89,"Y")/74)</f>
         <v/>
       </c>
     </row>
@@ -3577,15 +4011,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F26"/>
+  <dimension ref="B2:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="86" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="88" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -3598,14 +4032,14 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Carried across reps. A finding stays open until the rebuild produces it correctly without prompting.</t>
+          <t>A finding stays open until a rebuild produces it correctly without prompting.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Rep 1: 57/78   Rep 2: 72/78   Rep 3: 71/78 in 44 minutes</t>
+          <t>Rep 1: 57/78 Excel   Rep 2: 72/78 Excel   Rep 3: 71/78 Excel, 44 min   Rep 4: 70/78 on PAPER  (content only, out of 74: 57, 70, 69, 70)</t>
         </is>
       </c>
     </row>
@@ -3636,7 +4070,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="46" customHeight="1">
+    <row r="8" ht="52" customHeight="1">
       <c r="B8" s="17" t="inlineStr">
         <is>
           <t>1</t>
@@ -3659,11 +4093,11 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Now at B70 in current liabilities. This was your only repeat miss and it is closed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="46" customHeight="1">
+          <t>Fixed in rep 3, BROKEN AGAIN in rep 4. Three failures in four reps. You have the days driver, the working capital line and the cash flow change - every appearance is as a FLOW. The balance itself never gets a home in current liabilities. That is a conceptual tell, not a memory lapse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="52" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
         <is>
           <t>2</t>
@@ -3686,11 +4120,11 @@
       </c>
       <c r="F9" s="30" t="inlineStr">
         <is>
-          <t>B16 now reads 'Effective Tax Rate'. The rep 2 row said 'Effective interest rate' - it was the typing slip it looked like.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="46" customHeight="1">
+          <t>Present in reps 3 and 4. Closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="52" customHeight="1">
       <c r="B10" s="17" t="inlineStr">
         <is>
           <t>3</t>
@@ -3703,21 +4137,21 @@
       </c>
       <c r="D10" s="44" t="inlineStr">
         <is>
-          <t>IMPROVED</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="E10" s="17" t="inlineStr">
         <is>
-          <t>Debt schedule was too thin</t>
+          <t>Debt schedule too thin</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Now beginning / repayment / interest expense / ending. Still no draws-or-issuance line, so the roll-forward can only shrink: beginning - repayment = ending. Add the additions row.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="46" customHeight="1">
+          <t>Now beginning / increase-(decrease) / ending, plus the rate and interest expense, and you noted that short-term debt takes the same structure. That note is the right instinct - the pattern generalises.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
       <c r="B11" s="17" t="inlineStr">
         <is>
           <t>4</t>
@@ -3728,287 +4162,314 @@
           <t>Rep 3</t>
         </is>
       </c>
-      <c r="D11" s="33" t="inlineStr">
+      <c r="D11" s="44" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>Revolver schedule missing</t>
+        </is>
+      </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>Back as 'Debt Schedule 2' with minimum cash, rate, beginning, increase-(decrease), ending and interest expense. The sweep LOGIC (the MIN cap) is still not written down, but the structure is there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C12" s="43" t="inlineStr">
+        <is>
+          <t>Rep 3</t>
+        </is>
+      </c>
+      <c r="D12" s="44" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>Revolver rate and minimum cash assumptions dropped</t>
+        </is>
+      </c>
+      <c r="F12" s="30" t="inlineStr">
+        <is>
+          <t>Both back in rep 4. Closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="52" customHeight="1">
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C13" s="43" t="inlineStr">
+        <is>
+          <t>Rep 2</t>
+        </is>
+      </c>
+      <c r="D13" s="44" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>'Dividends' as a row inside shareholders' equity</t>
+        </is>
+      </c>
+      <c r="F13" s="30" t="inlineStr">
+        <is>
+          <t>Gone. Equity now reads Common Equity, Retained Earnings, Total Equity. Open for two reps - closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="52" customHeight="1">
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C14" s="43" t="inlineStr">
+        <is>
+          <t>Rep 2</t>
+        </is>
+      </c>
+      <c r="D14" s="44" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>No revolver line in cash flow financing</t>
+        </is>
+      </c>
+      <c r="F14" s="30" t="inlineStr">
+        <is>
+          <t>'Change in Revolver' now sits in financing alongside long-term debt, short-term debt, equity and dividends. Financing is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C15" s="43" t="inlineStr">
+        <is>
+          <t>Rep 4</t>
+        </is>
+      </c>
+      <c r="D15" s="33" t="inlineStr">
         <is>
           <t>REGRESSED</t>
         </is>
       </c>
-      <c r="E11" s="17" t="inlineStr">
-        <is>
-          <t>Revolver schedule is now an empty header</t>
-        </is>
-      </c>
-      <c r="F11" s="30" t="inlineStr">
-        <is>
-          <t>Rows 175-177 carry the title, the units note and the date row - and nothing else. Rep 2 had a working block with live draw and repayment formulas. It was not rebuilt this time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="46" customHeight="1">
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C12" s="43" t="inlineStr">
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>The entire PP&amp;E chain dropped out</t>
+        </is>
+      </c>
+      <c r="F15" s="30" t="inlineStr">
+        <is>
+          <t>No asset schedule anywhere in the seven pages, and no depreciation-as-a-%-of-PP&amp;E assumption. Both were present in reps 2 and 3. Depreciation still appears on the income statement, so it is the DRIVER and the SCHEDULE that went, not the concept - a single coherent omission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52" customHeight="1">
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C16" s="43" t="inlineStr">
+        <is>
+          <t>Rep 4</t>
+        </is>
+      </c>
+      <c r="D16" s="35" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>Equity schedule is better than before</t>
+        </is>
+      </c>
+      <c r="F16" s="30" t="inlineStr">
+        <is>
+          <t>Split into two roll-forwards - common equity, and retained earnings with net income and (dividends). That is more correct than the single block in rep 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="52" customHeight="1">
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C17" s="43" t="inlineStr">
+        <is>
+          <t>Rep 4</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="inlineStr">
+        <is>
+          <t>NIT</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>Investing subtotal mislabelled</t>
+        </is>
+      </c>
+      <c r="F17" s="30" t="inlineStr">
+        <is>
+          <t>Reads 'Net Change in Cash from Operating Activities' under the investing section. Copy error.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1">
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C18" s="43" t="inlineStr">
+        <is>
+          <t>Rep 2</t>
+        </is>
+      </c>
+      <c r="D18" s="45" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>No colour convention</t>
+        </is>
+      </c>
+      <c r="F18" s="30" t="inlineStr">
+        <is>
+          <t>Not scoreable on a paper rep. Still outstanding for the next Excel rep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="52" customHeight="1">
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C19" s="43" t="inlineStr">
+        <is>
+          <t>Rep 2</t>
+        </is>
+      </c>
+      <c r="D19" s="45" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>'Cash from Operations' header placement</t>
+        </is>
+      </c>
+      <c r="F19" s="30" t="inlineStr">
+        <is>
+          <t>On paper the section headers now read correctly. Re-check on the next Excel rep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="52" customHeight="1">
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C20" s="43" t="inlineStr">
         <is>
           <t>Rep 3</t>
         </is>
       </c>
-      <c r="D12" s="33" t="inlineStr">
-        <is>
-          <t>REGRESSED</t>
-        </is>
-      </c>
-      <c r="E12" s="17" t="inlineStr">
-        <is>
-          <t>Revolver rate and minimum cash assumptions dropped</t>
-        </is>
-      </c>
-      <c r="F12" s="30" t="inlineStr">
-        <is>
-          <t>Both were present in rep 2 and are gone from the assumptions block. Without a minimum cash balance the sweep has nothing to solve against.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="46" customHeight="1">
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C13" s="43" t="inlineStr">
-        <is>
-          <t>Rep 2</t>
-        </is>
-      </c>
-      <c r="D13" s="45" t="inlineStr">
+      <c r="D20" s="45" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="E13" s="17" t="inlineStr">
-        <is>
-          <t>'Dividends' still sits as a row inside shareholders' equity</t>
-        </is>
-      </c>
-      <c r="F13" s="30" t="inlineStr">
-        <is>
-          <t>B81. Flagged last rep, unchanged. Dividends are a flow - income statement, financing on the CFS, and a deduction inside the equity roll-forward. Not a balance sheet row.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="46" customHeight="1">
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C14" s="43" t="inlineStr">
-        <is>
-          <t>Rep 2</t>
-        </is>
-      </c>
-      <c r="D14" s="45" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E14" s="17" t="inlineStr">
-        <is>
-          <t>No revolver line in cash flow financing</t>
-        </is>
-      </c>
-      <c r="F14" s="30" t="inlineStr">
-        <is>
-          <t>Financing still has debt, equity and dividends only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="46" customHeight="1">
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C15" s="43" t="inlineStr">
-        <is>
-          <t>Rep 2</t>
-        </is>
-      </c>
-      <c r="D15" s="45" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E15" s="17" t="inlineStr">
-        <is>
-          <t>No colour convention anywhere</t>
-        </is>
-      </c>
-      <c r="F15" s="30" t="inlineStr">
-        <is>
-          <t>All 203 populated cells still use the default theme font. Blue inputs, black formulas, green cross-sheet links.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="46" customHeight="1">
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C16" s="43" t="inlineStr">
-        <is>
-          <t>Rep 2</t>
-        </is>
-      </c>
-      <c r="D16" s="45" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E16" s="17" t="inlineStr">
-        <is>
-          <t>'Cash from Operations' header sits below net income</t>
-        </is>
-      </c>
-      <c r="F16" s="30" t="inlineStr">
-        <is>
-          <t>B97, after net income and depreciation. Move it above so the section reads top-down.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="46" customHeight="1">
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C17" s="43" t="inlineStr">
-        <is>
-          <t>Rep 3</t>
-        </is>
-      </c>
-      <c r="D17" s="45" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E17" s="17" t="inlineStr">
-        <is>
-          <t>No actual vs. projected markers on the periods</t>
-        </is>
-      </c>
-      <c r="F17" s="30" t="inlineStr">
-        <is>
-          <t>Eight periods now run 2022 to 2029, but nothing says where history stops and the forecast starts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="46" customHeight="1">
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C18" s="43" t="inlineStr">
-        <is>
-          <t>Rep 3</t>
-        </is>
-      </c>
-      <c r="D18" s="35" t="inlineStr">
-        <is>
-          <t>NOTE</t>
-        </is>
-      </c>
-      <c r="E18" s="17" t="inlineStr">
-        <is>
-          <t>Day 2's layer was not attempted</t>
-        </is>
-      </c>
-      <c r="F18" s="30" t="inlineStr">
-        <is>
-          <t>The ladder's Day 2 is periods PLUS assumption values. There is not a single number in the file - this was another skeleton rep. Not wrong, but the layer is still outstanding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>NEXT REP - fix list, in order</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="23" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C21" s="25" t="inlineStr">
-        <is>
-          <t>Rebuild the revolver block and put its two assumptions back (findings 4 and 5).</t>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>Assumption VALUES still not attempted</t>
+        </is>
+      </c>
+      <c r="F20" s="30" t="inlineStr">
+        <is>
+          <t>Four reps, no numbers. The skeleton is close to automatic now - the Day 2 layer is overdue.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="23" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="C22" s="25" t="inlineStr">
-        <is>
-          <t>Delete the Dividends row from shareholders' equity (finding 6).</t>
+      <c r="B22" s="52" t="inlineStr">
+        <is>
+          <t>THE PATTERN</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="23" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C23" s="25" t="inlineStr">
-        <is>
-          <t>Add a revolver line to cash flow financing (finding 7).</t>
+      <c r="B23" s="31" t="inlineStr">
+        <is>
+          <t>Rep 2 to 3: fixed taxes payable and the tax rate - dropped the revolver block and two of its assumptions.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="23" t="inlineStr">
-        <is>
-          <t>4.</t>
-        </is>
-      </c>
-      <c r="C24" s="25" t="inlineStr">
-        <is>
-          <t>Add the draws row to the debt schedule (finding 3).</t>
+      <c r="B24" s="31" t="inlineStr">
+        <is>
+          <t>Rep 3 to 4: fixed the revolver, dividends-in-equity and financing - dropped the whole PP&amp;E chain, and taxes payable again.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="23" t="inlineStr">
-        <is>
-          <t>5.</t>
-        </is>
-      </c>
-      <c r="C25" s="25" t="inlineStr">
-        <is>
-          <t>Colour every cell as you type it - blue, black, green (finding 8).</t>
-        </is>
-      </c>
+      <c r="B25" s="31" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>6.</t>
-        </is>
-      </c>
-      <c r="C26" s="25" t="inlineStr">
-        <is>
-          <t>Then, and only then, enter assumption values. That is the Day 2 layer.</t>
+          <t>You are not forgetting things at random. Each rep, the fix list takes the attention that was holding the rest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="23" t="inlineStr">
+        <is>
+          <t>The answer is not to try harder on recall. Add a CLOSING SWEEP: when the skeleton feels finished, spend three</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="23" t="inlineStr">
+        <is>
+          <t>minutes walking the four schedules and the balance sheet against a fixed order before calling it done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>Verification is a much easier task than recall, and it catches exactly this failure.</t>
         </is>
       </c>
     </row>
@@ -4289,7 +4750,7 @@
       </c>
       <c r="E9" s="30" t="inlineStr">
         <is>
-          <t>Skeleton rebuilt in 44 min at 71/78. Balance sheet perfect, tax rate and taxes-payable fixed. Revolver block and its assumptions regressed. Assumption VALUES still outstanding - repeat Day 2.</t>
+          <t>Four skeleton reps done. Rep 4 on paper: 70/74 on content, tied with the best. Seven findings closed. PP&amp;E chain and income taxes payable are the live gaps. Assumption VALUES still outstanding.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Score rep 5 and add the Larkfield practice report
Rep 5 scores 73/78, the best yet and the first rep with all four
schedules and a complete balance sheet together. Income taxes payable
and the PP&E chain are both present, and the revolver draw and repay
formulas now carry the correct MIN cap.

One bug recorded: the revolver ending balance sums beginning, draw and
repayment while the repayment is computed positive, so the balance grows
when it should shrink. Wrong in three of six stress cases; the chosen
test case is a draw year, which hides it.

Adds a fictional three-year financial report to model from, plus the
generator that builds it. The figures are constructed so the balance
sheet balances in every period, the cash flow statement reconciles to
balance sheet cash, and the working capital, fixed asset and equity
movements are internally consistent.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UX5HPwj2AEakAb4LMEQ7Bv
</commit_message>
<xml_diff>
--- a/learning/model-practice/Day_2_scorecard_and_ladder.xlsx
+++ b/learning/model-practice/Day_2_scorecard_and_ladder.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="29">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -191,6 +191,18 @@
       <color rgb="FFC00000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF008000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1546C9"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -256,7 +268,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -354,6 +366,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -787,6 +801,11 @@
           <t>Paper</t>
         </is>
       </c>
+      <c r="I5" s="47" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
@@ -973,7 +992,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I11" s="13" t="n"/>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J11" s="13" t="n"/>
       <c r="K11" s="13" t="n"/>
     </row>
@@ -1005,7 +1028,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I12" s="13" t="n"/>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J12" s="13" t="n"/>
       <c r="K12" s="13" t="n"/>
     </row>
@@ -1037,7 +1064,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I13" s="13" t="n"/>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J13" s="13" t="n"/>
       <c r="K13" s="13" t="n"/>
     </row>
@@ -1069,7 +1100,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I14" s="13" t="n"/>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J14" s="13" t="n"/>
       <c r="K14" s="13" t="n"/>
     </row>
@@ -1105,7 +1140,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I15" s="13" t="n"/>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J15" s="13" t="n"/>
       <c r="K15" s="13" t="n"/>
     </row>
@@ -1137,7 +1176,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I16" s="13" t="n"/>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J16" s="13" t="n"/>
       <c r="K16" s="13" t="n"/>
     </row>
@@ -1169,7 +1212,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I17" s="13" t="n"/>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J17" s="13" t="n"/>
       <c r="K17" s="13" t="n"/>
     </row>
@@ -1201,7 +1248,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I18" s="13" t="n"/>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J18" s="13" t="n"/>
       <c r="K18" s="13" t="n"/>
     </row>
@@ -1233,7 +1284,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I19" s="13" t="n"/>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J19" s="13" t="n"/>
       <c r="K19" s="13" t="n"/>
     </row>
@@ -1269,7 +1324,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I20" s="13" t="n"/>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J20" s="13" t="n"/>
       <c r="K20" s="13" t="n"/>
     </row>
@@ -1301,7 +1360,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I21" s="13" t="n"/>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J21" s="13" t="n"/>
       <c r="K21" s="13" t="n"/>
     </row>
@@ -1333,7 +1396,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I22" s="13" t="n"/>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J22" s="13" t="n"/>
       <c r="K22" s="13" t="n"/>
     </row>
@@ -1369,7 +1436,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I23" s="13" t="n"/>
+      <c r="I23" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J23" s="13" t="n"/>
       <c r="K23" s="13" t="n"/>
     </row>
@@ -1405,7 +1476,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I24" s="13" t="n"/>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J24" s="13" t="n"/>
       <c r="K24" s="13" t="n"/>
     </row>
@@ -1441,7 +1516,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I25" s="13" t="n"/>
+      <c r="I25" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="J25" s="13" t="n"/>
       <c r="K25" s="13" t="n"/>
     </row>
@@ -1473,7 +1552,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I26" s="13" t="n"/>
+      <c r="I26" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="J26" s="13" t="n"/>
       <c r="K26" s="13" t="n"/>
     </row>
@@ -1505,7 +1588,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I27" s="13" t="n"/>
+      <c r="I27" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J27" s="13" t="n"/>
       <c r="K27" s="13" t="n"/>
     </row>
@@ -1537,7 +1624,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I28" s="13" t="n"/>
+      <c r="I28" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J28" s="13" t="n"/>
       <c r="K28" s="13" t="n"/>
     </row>
@@ -1585,7 +1676,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I30" s="13" t="n"/>
+      <c r="I30" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J30" s="13" t="n"/>
       <c r="K30" s="13" t="n"/>
     </row>
@@ -1617,7 +1712,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I31" s="13" t="n"/>
+      <c r="I31" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J31" s="13" t="n"/>
       <c r="K31" s="13" t="n"/>
     </row>
@@ -1653,7 +1752,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I32" s="13" t="n"/>
+      <c r="I32" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J32" s="13" t="n"/>
       <c r="K32" s="13" t="n"/>
     </row>
@@ -1685,7 +1788,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I33" s="13" t="n"/>
+      <c r="I33" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J33" s="13" t="n"/>
       <c r="K33" s="13" t="n"/>
     </row>
@@ -1717,7 +1824,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I34" s="13" t="n"/>
+      <c r="I34" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J34" s="13" t="n"/>
       <c r="K34" s="13" t="n"/>
     </row>
@@ -1749,7 +1860,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I35" s="13" t="n"/>
+      <c r="I35" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J35" s="13" t="n"/>
       <c r="K35" s="13" t="n"/>
     </row>
@@ -1781,7 +1896,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I36" s="13" t="n"/>
+      <c r="I36" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J36" s="13" t="n"/>
       <c r="K36" s="13" t="n"/>
     </row>
@@ -1813,7 +1932,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I37" s="13" t="n"/>
+      <c r="I37" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J37" s="13" t="n"/>
       <c r="K37" s="13" t="n"/>
     </row>
@@ -1849,7 +1972,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I38" s="13" t="n"/>
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J38" s="13" t="n"/>
       <c r="K38" s="13" t="n"/>
     </row>
@@ -1881,7 +2008,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I39" s="13" t="n"/>
+      <c r="I39" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J39" s="13" t="n"/>
       <c r="K39" s="13" t="n"/>
     </row>
@@ -1913,7 +2044,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I40" s="13" t="n"/>
+      <c r="I40" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J40" s="13" t="n"/>
       <c r="K40" s="13" t="n"/>
     </row>
@@ -1945,7 +2080,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I41" s="13" t="n"/>
+      <c r="I41" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J41" s="13" t="n"/>
       <c r="K41" s="13" t="n"/>
     </row>
@@ -1977,7 +2116,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I42" s="13" t="n"/>
+      <c r="I42" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J42" s="13" t="n"/>
       <c r="K42" s="13" t="n"/>
     </row>
@@ -2009,7 +2152,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I43" s="13" t="n"/>
+      <c r="I43" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J43" s="13" t="n"/>
       <c r="K43" s="13" t="n"/>
     </row>
@@ -2057,7 +2204,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I45" s="13" t="n"/>
+      <c r="I45" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J45" s="13" t="n"/>
       <c r="K45" s="13" t="n"/>
     </row>
@@ -2089,7 +2240,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I46" s="13" t="n"/>
+      <c r="I46" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J46" s="13" t="n"/>
       <c r="K46" s="13" t="n"/>
     </row>
@@ -2121,7 +2276,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I47" s="13" t="n"/>
+      <c r="I47" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J47" s="13" t="n"/>
       <c r="K47" s="13" t="n"/>
     </row>
@@ -2157,7 +2316,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I48" s="13" t="n"/>
+      <c r="I48" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J48" s="13" t="n"/>
       <c r="K48" s="13" t="n"/>
     </row>
@@ -2189,7 +2352,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I49" s="13" t="n"/>
+      <c r="I49" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J49" s="13" t="n"/>
       <c r="K49" s="13" t="n"/>
     </row>
@@ -2221,7 +2388,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I50" s="13" t="n"/>
+      <c r="I50" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J50" s="13" t="n"/>
       <c r="K50" s="13" t="n"/>
     </row>
@@ -2253,7 +2424,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I51" s="13" t="n"/>
+      <c r="I51" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J51" s="13" t="n"/>
       <c r="K51" s="13" t="n"/>
     </row>
@@ -2285,7 +2460,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I52" s="13" t="n"/>
+      <c r="I52" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J52" s="13" t="n"/>
       <c r="K52" s="13" t="n"/>
     </row>
@@ -2317,7 +2496,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I53" s="13" t="n"/>
+      <c r="I53" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J53" s="13" t="n"/>
       <c r="K53" s="13" t="n"/>
     </row>
@@ -2353,7 +2536,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I54" s="13" t="n"/>
+      <c r="I54" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J54" s="13" t="n"/>
       <c r="K54" s="13" t="n"/>
     </row>
@@ -2385,7 +2572,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I55" s="13" t="n"/>
+      <c r="I55" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J55" s="13" t="n"/>
       <c r="K55" s="13" t="n"/>
     </row>
@@ -2417,7 +2608,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I56" s="13" t="n"/>
+      <c r="I56" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J56" s="13" t="n"/>
       <c r="K56" s="13" t="n"/>
     </row>
@@ -2453,7 +2648,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I57" s="13" t="n"/>
+      <c r="I57" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J57" s="13" t="n"/>
       <c r="K57" s="13" t="n"/>
     </row>
@@ -2485,7 +2684,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I58" s="13" t="n"/>
+      <c r="I58" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J58" s="13" t="n"/>
       <c r="K58" s="13" t="n"/>
     </row>
@@ -2517,7 +2720,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I59" s="13" t="n"/>
+      <c r="I59" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J59" s="13" t="n"/>
       <c r="K59" s="13" t="n"/>
     </row>
@@ -2549,7 +2756,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I60" s="13" t="n"/>
+      <c r="I60" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J60" s="13" t="n"/>
       <c r="K60" s="13" t="n"/>
     </row>
@@ -2581,7 +2792,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I61" s="13" t="n"/>
+      <c r="I61" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J61" s="13" t="n"/>
       <c r="K61" s="13" t="n"/>
     </row>
@@ -2613,7 +2828,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I62" s="13" t="n"/>
+      <c r="I62" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J62" s="13" t="n"/>
       <c r="K62" s="13" t="n"/>
     </row>
@@ -2645,7 +2864,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I63" s="13" t="n"/>
+      <c r="I63" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J63" s="13" t="n"/>
       <c r="K63" s="13" t="n"/>
     </row>
@@ -2681,7 +2904,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I64" s="13" t="n"/>
+      <c r="I64" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J64" s="13" t="n"/>
       <c r="K64" s="13" t="n"/>
     </row>
@@ -2729,7 +2956,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I66" s="13" t="n"/>
+      <c r="I66" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J66" s="13" t="n"/>
       <c r="K66" s="13" t="n"/>
     </row>
@@ -2761,7 +2992,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I67" s="13" t="n"/>
+      <c r="I67" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J67" s="13" t="n"/>
       <c r="K67" s="13" t="n"/>
     </row>
@@ -2793,7 +3028,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I68" s="13" t="n"/>
+      <c r="I68" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J68" s="13" t="n"/>
       <c r="K68" s="13" t="n"/>
     </row>
@@ -2825,7 +3064,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I69" s="13" t="n"/>
+      <c r="I69" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J69" s="13" t="n"/>
       <c r="K69" s="13" t="n"/>
     </row>
@@ -2857,7 +3100,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I70" s="13" t="n"/>
+      <c r="I70" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J70" s="13" t="n"/>
       <c r="K70" s="13" t="n"/>
     </row>
@@ -2889,7 +3136,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I71" s="13" t="n"/>
+      <c r="I71" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J71" s="13" t="n"/>
       <c r="K71" s="13" t="n"/>
     </row>
@@ -2921,7 +3172,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I72" s="13" t="n"/>
+      <c r="I72" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J72" s="13" t="n"/>
       <c r="K72" s="13" t="n"/>
     </row>
@@ -2953,7 +3208,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I73" s="13" t="n"/>
+      <c r="I73" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J73" s="13" t="n"/>
       <c r="K73" s="13" t="n"/>
     </row>
@@ -2985,7 +3244,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I74" s="13" t="n"/>
+      <c r="I74" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J74" s="13" t="n"/>
       <c r="K74" s="13" t="n"/>
     </row>
@@ -3017,7 +3280,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I75" s="13" t="n"/>
+      <c r="I75" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J75" s="13" t="n"/>
       <c r="K75" s="13" t="n"/>
     </row>
@@ -3049,7 +3316,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I76" s="13" t="n"/>
+      <c r="I76" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="J76" s="13" t="n"/>
       <c r="K76" s="13" t="n"/>
     </row>
@@ -3081,7 +3352,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I77" s="13" t="n"/>
+      <c r="I77" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J77" s="13" t="n"/>
       <c r="K77" s="13" t="n"/>
     </row>
@@ -3117,7 +3392,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I78" s="13" t="n"/>
+      <c r="I78" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J78" s="13" t="n"/>
       <c r="K78" s="13" t="n"/>
     </row>
@@ -3149,7 +3428,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I79" s="13" t="n"/>
+      <c r="I79" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J79" s="13" t="n"/>
       <c r="K79" s="13" t="n"/>
     </row>
@@ -3181,7 +3464,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I80" s="13" t="n"/>
+      <c r="I80" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J80" s="13" t="n"/>
       <c r="K80" s="13" t="n"/>
     </row>
@@ -3213,7 +3500,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I81" s="13" t="n"/>
+      <c r="I81" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J81" s="13" t="n"/>
       <c r="K81" s="13" t="n"/>
     </row>
@@ -3245,7 +3536,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I82" s="13" t="n"/>
+      <c r="I82" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J82" s="13" t="n"/>
       <c r="K82" s="13" t="n"/>
     </row>
@@ -3297,7 +3592,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I84" s="13" t="n"/>
+      <c r="I84" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J84" s="13" t="n"/>
       <c r="K84" s="13" t="n"/>
     </row>
@@ -3329,7 +3628,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I85" s="13" t="n"/>
+      <c r="I85" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J85" s="13" t="n"/>
       <c r="K85" s="13" t="n"/>
     </row>
@@ -3361,7 +3664,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I86" s="13" t="n"/>
+      <c r="I86" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J86" s="13" t="n"/>
       <c r="K86" s="13" t="n"/>
     </row>
@@ -3393,7 +3700,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I87" s="13" t="n"/>
+      <c r="I87" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J87" s="13" t="n"/>
       <c r="K87" s="13" t="n"/>
     </row>
@@ -3425,7 +3736,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I88" s="13" t="n"/>
+      <c r="I88" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J88" s="13" t="n"/>
       <c r="K88" s="13" t="n"/>
     </row>
@@ -3477,7 +3792,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I90" s="13" t="n"/>
+      <c r="I90" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J90" s="13" t="n"/>
       <c r="K90" s="13" t="n"/>
     </row>
@@ -3509,7 +3828,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I91" s="13" t="n"/>
+      <c r="I91" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="J91" s="13" t="n"/>
       <c r="K91" s="13" t="n"/>
     </row>
@@ -3541,7 +3864,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I92" s="13" t="n"/>
+      <c r="I92" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="J92" s="13" t="n"/>
       <c r="K92" s="13" t="n"/>
     </row>
@@ -3573,7 +3900,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I93" s="13" t="n"/>
+      <c r="I93" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="J93" s="13" t="n"/>
       <c r="K93" s="13" t="n"/>
     </row>
@@ -4011,15 +4342,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F29"/>
+  <dimension ref="B2:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="88" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="92" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -4029,447 +4360,335 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>A finding stays open until a rebuild produces it correctly without prompting.</t>
-        </is>
-      </c>
-    </row>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Rep 1: 57/78 Excel   Rep 2: 72/78 Excel   Rep 3: 71/78 Excel, 44 min   Rep 4: 70/78 on PAPER  (content only, out of 74: 57, 70, 69, 70)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="6" t="inlineStr">
+          <t>Rep 1: 57   Rep 2: 72   Rep 3: 71   Rep 4: 70 (paper)   Rep 5: 73 / 78     content only /74:  57 · 70 · 69 · 70 · 71</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="53" t="inlineStr">
+        <is>
+          <t>Rep 5 is the best score yet, and the first with all four schedules AND a complete balance sheet in the same rep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Since</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Finding</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="52" customHeight="1">
-      <c r="B8" s="17" t="inlineStr">
+    <row r="9" ht="54" customHeight="1">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C8" s="43" t="inlineStr">
+      <c r="C9" s="43" t="inlineStr">
         <is>
           <t>Rep 2</t>
         </is>
       </c>
-      <c r="D8" s="44" t="inlineStr">
+      <c r="D9" s="44" t="inlineStr">
         <is>
           <t>FIXED</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
-        <is>
-          <t>Income taxes payable absent from the balance sheet</t>
-        </is>
-      </c>
-      <c r="F8" s="30" t="inlineStr">
-        <is>
-          <t>Fixed in rep 3, BROKEN AGAIN in rep 4. Three failures in four reps. You have the days driver, the working capital line and the cash flow change - every appearance is as a FLOW. The balance itself never gets a home in current liabilities. That is a conceptual tell, not a memory lapse.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="B9" s="17" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>Income taxes payable on the balance sheet</t>
+        </is>
+      </c>
+      <c r="F9" s="30" t="inlineStr">
+        <is>
+          <t>B73, in current liabilities. Failed three of the first four reps - present in rep 5. This was the big one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C9" s="43" t="inlineStr">
+      <c r="C10" s="43" t="inlineStr">
+        <is>
+          <t>Rep 4</t>
+        </is>
+      </c>
+      <c r="D10" s="44" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>The PP&amp;E chain</t>
+        </is>
+      </c>
+      <c r="F10" s="30" t="inlineStr">
+        <is>
+          <t>Asset schedule back at B196-199 as a proper roll-forward, and the depreciation-as-%-of-PP&amp;E driver back at B10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1">
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C11" s="43" t="inlineStr">
         <is>
           <t>Rep 2</t>
         </is>
       </c>
-      <c r="D9" s="44" t="inlineStr">
+      <c r="D11" s="44" t="inlineStr">
         <is>
           <t>FIXED</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>No effective tax rate assumption</t>
-        </is>
-      </c>
-      <c r="F9" s="30" t="inlineStr">
-        <is>
-          <t>Present in reps 3 and 4. Closed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="52" customHeight="1">
-      <c r="B10" s="17" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C10" s="43" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>Debt schedule</t>
+        </is>
+      </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>Best version yet: long-term and short-term modelled separately, each with beginning, increase-(repayment), ending, its own rate and its own interest expense line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1">
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C12" s="43" t="inlineStr">
         <is>
           <t>Rep 2</t>
         </is>
       </c>
-      <c r="D10" s="44" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="E10" s="17" t="inlineStr">
-        <is>
-          <t>Debt schedule too thin</t>
-        </is>
-      </c>
-      <c r="F10" s="30" t="inlineStr">
-        <is>
-          <t>Now beginning / increase-(decrease) / ending, plus the rate and interest expense, and you noted that short-term debt takes the same structure. That note is the right instinct - the pattern generalises.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="52" customHeight="1">
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>Revolver ending balance ADDS the repayment</t>
+        </is>
+      </c>
+      <c r="F12" s="30">
+        <f>SUM(E178:E180) sums beginning + draw + repayment, but the repayment is computed as a POSITIVE number - so the revolver GROWS when it should shrink. Wrong in 3 of 6 stress cases: begin 40, cash 200, min 140 gives 80 where it should give 0. Fix: make the repayment negative, =-MAX(MIN(E173-E176,E178),0), and keep the SUM.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1">
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C13" s="43" t="inlineStr">
+        <is>
+          <t>Rep 5</t>
+        </is>
+      </c>
+      <c r="D13" s="35" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>The draw and repay LOGIC is now correct</t>
+        </is>
+      </c>
+      <c r="F13" s="30">
+        <f>MAX(E176-E173,0) and =MAX(MIN(E173-E176,E178),0). The MIN cap that was missing in rep 2 is there and correct in every stress case. Only the sign on the ending line is wrong.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1">
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C14" s="43" t="inlineStr">
+        <is>
+          <t>Rep 5</t>
+        </is>
+      </c>
+      <c r="D14" s="35" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>Your test case hides the bug - again</t>
+        </is>
+      </c>
+      <c r="F14" s="30" t="inlineStr">
+        <is>
+          <t>Cash 120 against a 140 minimum is a DRAW year, so the repayment is zero and the sign error cannot show. Rep 2 had exactly the same blind spot. When you test a sweep, always test a repayment year too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1">
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C15" s="43" t="inlineStr">
+        <is>
+          <t>Rep 5</t>
+        </is>
+      </c>
+      <c r="D15" s="33" t="inlineStr">
+        <is>
+          <t>REGRESSED</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>Dividends as a % of net income dropped from assumptions</t>
+        </is>
+      </c>
+      <c r="F15" s="30" t="inlineStr">
+        <is>
+          <t>Present in reps 1 through 4. The Dividends line is still on the income statement and in both the cash flow and the equity schedule - only the driver went.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1">
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C16" s="43" t="inlineStr">
+        <is>
+          <t>Rep 4</t>
+        </is>
+      </c>
+      <c r="D16" s="33" t="inlineStr">
+        <is>
+          <t>REGRESSED</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>No revolver line in cash flow financing</t>
+        </is>
+      </c>
+      <c r="F16" s="30" t="inlineStr">
+        <is>
+          <t>You had it in rep 4. Financing is back to debt, equity and dividends only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1">
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C17" s="43" t="inlineStr">
+        <is>
+          <t>Rep 2</t>
+        </is>
+      </c>
+      <c r="D17" s="45" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>No colour convention</t>
+        </is>
+      </c>
+      <c r="F17" s="30" t="inlineStr">
+        <is>
+          <t>All 230 populated cells still default theme font. This is the last easy structural win.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1">
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C18" s="43" t="inlineStr">
         <is>
           <t>Rep 3</t>
         </is>
       </c>
-      <c r="D11" s="44" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="E11" s="17" t="inlineStr">
-        <is>
-          <t>Revolver schedule missing</t>
-        </is>
-      </c>
-      <c r="F11" s="30" t="inlineStr">
-        <is>
-          <t>Back as 'Debt Schedule 2' with minimum cash, rate, beginning, increase-(decrease), ending and interest expense. The sweep LOGIC (the MIN cap) is still not written down, but the structure is there.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="52" customHeight="1">
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C12" s="43" t="inlineStr">
+      <c r="D18" s="45" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>No actual vs projected markers</t>
+        </is>
+      </c>
+      <c r="F18" s="30" t="inlineStr"/>
+    </row>
+    <row r="19" ht="54" customHeight="1">
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C19" s="43" t="inlineStr">
         <is>
           <t>Rep 3</t>
         </is>
       </c>
-      <c r="D12" s="44" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="E12" s="17" t="inlineStr">
-        <is>
-          <t>Revolver rate and minimum cash assumptions dropped</t>
-        </is>
-      </c>
-      <c r="F12" s="30" t="inlineStr">
-        <is>
-          <t>Both back in rep 4. Closed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="52" customHeight="1">
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C13" s="43" t="inlineStr">
-        <is>
-          <t>Rep 2</t>
-        </is>
-      </c>
-      <c r="D13" s="44" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="E13" s="17" t="inlineStr">
-        <is>
-          <t>'Dividends' as a row inside shareholders' equity</t>
-        </is>
-      </c>
-      <c r="F13" s="30" t="inlineStr">
-        <is>
-          <t>Gone. Equity now reads Common Equity, Retained Earnings, Total Equity. Open for two reps - closed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="52" customHeight="1">
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C14" s="43" t="inlineStr">
-        <is>
-          <t>Rep 2</t>
-        </is>
-      </c>
-      <c r="D14" s="44" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="E14" s="17" t="inlineStr">
-        <is>
-          <t>No revolver line in cash flow financing</t>
-        </is>
-      </c>
-      <c r="F14" s="30" t="inlineStr">
-        <is>
-          <t>'Change in Revolver' now sits in financing alongside long-term debt, short-term debt, equity and dividends. Financing is complete.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="52" customHeight="1">
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C15" s="43" t="inlineStr">
-        <is>
-          <t>Rep 4</t>
-        </is>
-      </c>
-      <c r="D15" s="33" t="inlineStr">
-        <is>
-          <t>REGRESSED</t>
-        </is>
-      </c>
-      <c r="E15" s="17" t="inlineStr">
-        <is>
-          <t>The entire PP&amp;E chain dropped out</t>
-        </is>
-      </c>
-      <c r="F15" s="30" t="inlineStr">
-        <is>
-          <t>No asset schedule anywhere in the seven pages, and no depreciation-as-a-%-of-PP&amp;E assumption. Both were present in reps 2 and 3. Depreciation still appears on the income statement, so it is the DRIVER and the SCHEDULE that went, not the concept - a single coherent omission.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="52" customHeight="1">
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C16" s="43" t="inlineStr">
-        <is>
-          <t>Rep 4</t>
-        </is>
-      </c>
-      <c r="D16" s="35" t="inlineStr">
-        <is>
-          <t>NOTE</t>
-        </is>
-      </c>
-      <c r="E16" s="17" t="inlineStr">
-        <is>
-          <t>Equity schedule is better than before</t>
-        </is>
-      </c>
-      <c r="F16" s="30" t="inlineStr">
-        <is>
-          <t>Split into two roll-forwards - common equity, and retained earnings with net income and (dividends). That is more correct than the single block in rep 3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="52" customHeight="1">
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C17" s="43" t="inlineStr">
-        <is>
-          <t>Rep 4</t>
-        </is>
-      </c>
-      <c r="D17" s="35" t="inlineStr">
-        <is>
-          <t>NIT</t>
-        </is>
-      </c>
-      <c r="E17" s="17" t="inlineStr">
-        <is>
-          <t>Investing subtotal mislabelled</t>
-        </is>
-      </c>
-      <c r="F17" s="30" t="inlineStr">
-        <is>
-          <t>Reads 'Net Change in Cash from Operating Activities' under the investing section. Copy error.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="52" customHeight="1">
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C18" s="43" t="inlineStr">
-        <is>
-          <t>Rep 2</t>
-        </is>
-      </c>
-      <c r="D18" s="45" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E18" s="17" t="inlineStr">
-        <is>
-          <t>No colour convention</t>
-        </is>
-      </c>
-      <c r="F18" s="30" t="inlineStr">
-        <is>
-          <t>Not scoreable on a paper rep. Still outstanding for the next Excel rep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="52" customHeight="1">
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C19" s="43" t="inlineStr">
-        <is>
-          <t>Rep 2</t>
-        </is>
-      </c>
-      <c r="D19" s="45" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="D19" s="44" t="inlineStr">
+        <is>
+          <t>CLOSING</t>
         </is>
       </c>
       <c r="E19" s="17" t="inlineStr">
         <is>
-          <t>'Cash from Operations' header placement</t>
+          <t>Assumption values</t>
         </is>
       </c>
       <c r="F19" s="30" t="inlineStr">
         <is>
-          <t>On paper the section headers now read correctly. Re-check on the next Excel rep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="52" customHeight="1">
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="C20" s="43" t="inlineStr">
-        <is>
-          <t>Rep 3</t>
-        </is>
-      </c>
-      <c r="D20" s="45" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E20" s="17" t="inlineStr">
-        <is>
-          <t>Assumption VALUES still not attempted</t>
-        </is>
-      </c>
-      <c r="F20" s="30" t="inlineStr">
-        <is>
-          <t>Four reps, no numbers. The skeleton is close to automatic now - the Day 2 layer is overdue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="52" t="inlineStr">
-        <is>
-          <t>THE PATTERN</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="31" t="inlineStr">
-        <is>
-          <t>Rep 2 to 3: fixed taxes payable and the tax rate - dropped the revolver block and two of its assumptions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="31" t="inlineStr">
-        <is>
-          <t>Rep 3 to 4: fixed the revolver, dividends-in-equity and financing - dropped the whole PP&amp;E chain, and taxes payable again.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="31" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="23" t="inlineStr">
-        <is>
-          <t>You are not forgetting things at random. Each rep, the fix list takes the attention that was holding the rest.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="23" t="inlineStr">
-        <is>
-          <t>The answer is not to try harder on recall. Add a CLOSING SWEEP: when the skeleton feels finished, spend three</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="23" t="inlineStr">
-        <is>
-          <t>minutes walking the four schedules and the balance sheet against a fixed order before calling it done.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="23" t="inlineStr">
-        <is>
-          <t>Verification is a much easier task than recall, and it catches exactly this failure.</t>
+          <t>Five reps, no numbers. Resolved now - the fake report is the input for the next rep.</t>
         </is>
       </c>
     </row>
@@ -4738,9 +4957,9 @@
           <t>Day 2</t>
         </is>
       </c>
-      <c r="C9" s="46" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D9" s="17" t="inlineStr">
@@ -4750,7 +4969,7 @@
       </c>
       <c r="E9" s="30" t="inlineStr">
         <is>
-          <t>Four skeleton reps done. Rep 4 on paper: 70/74 on content, tied with the best. Seven findings closed. PP&amp;E chain and income taxes payable are the live gaps. Assumption VALUES still outstanding.</t>
+          <t>Skeleton is essentially automatic: 73/78, all four schedules, complete balance sheet, working MIN/MAX draw and repay logic. Move to Day 3 - put real numbers in from the Larkfield report.</t>
         </is>
       </c>
     </row>
@@ -4760,7 +4979,11 @@
           <t>Day 3</t>
         </is>
       </c>
-      <c r="C10" s="29" t="inlineStr"/>
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t>NEXT</t>
+        </is>
+      </c>
       <c r="D10" s="17" t="inlineStr">
         <is>
           <t>Income statement</t>

</xml_diff>

<commit_message>
Score rep 6 of the skeleton drill
Scores 72/78. Cash flow is complete for the second rep running and the
balance check now carries live formulas, the first computational content
in any skeleton attempt. The rep also adds blocks read out of the
Larkfield notes rather than recalled: a costs schedule driven by an
inflation rate, a revolver commitment fee, and short-term debt terms.

Records that the skeleton has converged. Five consecutive reps sit
between 69 and 71 of the 74 content items, so further structural
repetition has stopped paying; the remaining misses are small enough for
a closing sweep to catch. Marks entering numbers as the next step.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UX5HPwj2AEakAb4LMEQ7Bv
</commit_message>
<xml_diff>
--- a/learning/model-practice/Day_2_scorecard_and_ladder.xlsx
+++ b/learning/model-practice/Day_2_scorecard_and_ladder.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="31">
+  <fonts count="33">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -203,6 +203,18 @@
       <color rgb="FF1546C9"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FFB26B00"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFC00000"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -268,7 +280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -368,6 +380,9 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -806,6 +821,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="J5" s="47" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
@@ -997,7 +1017,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J11" s="13" t="n"/>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K11" s="13" t="n"/>
     </row>
     <row r="12">
@@ -1033,7 +1057,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J12" s="13" t="n"/>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K12" s="13" t="n"/>
     </row>
     <row r="13">
@@ -1069,7 +1097,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J13" s="13" t="n"/>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K13" s="13" t="n"/>
     </row>
     <row r="14">
@@ -1105,7 +1137,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J14" s="13" t="n"/>
+      <c r="J14" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K14" s="13" t="n"/>
     </row>
     <row r="15">
@@ -1145,7 +1181,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J15" s="13" t="n"/>
+      <c r="J15" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K15" s="13" t="n"/>
     </row>
     <row r="16">
@@ -1181,7 +1221,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J16" s="13" t="n"/>
+      <c r="J16" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K16" s="13" t="n"/>
     </row>
     <row r="17">
@@ -1217,7 +1261,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J17" s="13" t="n"/>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K17" s="13" t="n"/>
     </row>
     <row r="18">
@@ -1253,7 +1301,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J18" s="13" t="n"/>
+      <c r="J18" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K18" s="13" t="n"/>
     </row>
     <row r="19">
@@ -1289,7 +1341,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J19" s="13" t="n"/>
+      <c r="J19" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K19" s="13" t="n"/>
     </row>
     <row r="20">
@@ -1329,7 +1385,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J20" s="13" t="n"/>
+      <c r="J20" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K20" s="13" t="n"/>
     </row>
     <row r="21">
@@ -1365,7 +1425,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J21" s="13" t="n"/>
+      <c r="J21" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K21" s="13" t="n"/>
     </row>
     <row r="22">
@@ -1401,7 +1465,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J22" s="13" t="n"/>
+      <c r="J22" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K22" s="13" t="n"/>
     </row>
     <row r="23">
@@ -1441,7 +1509,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J23" s="13" t="n"/>
+      <c r="J23" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K23" s="13" t="n"/>
     </row>
     <row r="24">
@@ -1481,7 +1553,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J24" s="13" t="n"/>
+      <c r="J24" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="K24" s="13" t="n"/>
     </row>
     <row r="25">
@@ -1521,7 +1597,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J25" s="13" t="n"/>
+      <c r="J25" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="K25" s="13" t="n"/>
     </row>
     <row r="26">
@@ -1557,7 +1637,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J26" s="13" t="n"/>
+      <c r="J26" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="K26" s="13" t="n"/>
     </row>
     <row r="27">
@@ -1593,7 +1677,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J27" s="13" t="n"/>
+      <c r="J27" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K27" s="13" t="n"/>
     </row>
     <row r="28">
@@ -1629,7 +1717,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J28" s="13" t="n"/>
+      <c r="J28" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K28" s="13" t="n"/>
     </row>
     <row r="29">
@@ -1681,7 +1773,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J30" s="13" t="n"/>
+      <c r="J30" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K30" s="13" t="n"/>
     </row>
     <row r="31">
@@ -1717,7 +1813,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J31" s="13" t="n"/>
+      <c r="J31" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K31" s="13" t="n"/>
     </row>
     <row r="32">
@@ -1757,7 +1857,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J32" s="13" t="n"/>
+      <c r="J32" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K32" s="13" t="n"/>
     </row>
     <row r="33">
@@ -1793,7 +1897,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J33" s="13" t="n"/>
+      <c r="J33" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K33" s="13" t="n"/>
     </row>
     <row r="34">
@@ -1829,7 +1937,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J34" s="13" t="n"/>
+      <c r="J34" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K34" s="13" t="n"/>
     </row>
     <row r="35">
@@ -1865,7 +1977,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J35" s="13" t="n"/>
+      <c r="J35" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K35" s="13" t="n"/>
     </row>
     <row r="36">
@@ -1901,7 +2017,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J36" s="13" t="n"/>
+      <c r="J36" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K36" s="13" t="n"/>
     </row>
     <row r="37">
@@ -1937,7 +2057,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J37" s="13" t="n"/>
+      <c r="J37" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K37" s="13" t="n"/>
     </row>
     <row r="38">
@@ -1977,7 +2101,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J38" s="13" t="n"/>
+      <c r="J38" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K38" s="13" t="n"/>
     </row>
     <row r="39">
@@ -2013,7 +2141,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J39" s="13" t="n"/>
+      <c r="J39" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K39" s="13" t="n"/>
     </row>
     <row r="40">
@@ -2049,7 +2181,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J40" s="13" t="n"/>
+      <c r="J40" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K40" s="13" t="n"/>
     </row>
     <row r="41">
@@ -2085,7 +2221,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J41" s="13" t="n"/>
+      <c r="J41" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K41" s="13" t="n"/>
     </row>
     <row r="42">
@@ -2121,7 +2261,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J42" s="13" t="n"/>
+      <c r="J42" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K42" s="13" t="n"/>
     </row>
     <row r="43">
@@ -2157,7 +2301,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J43" s="13" t="n"/>
+      <c r="J43" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K43" s="13" t="n"/>
     </row>
     <row r="44">
@@ -2209,7 +2357,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J45" s="13" t="n"/>
+      <c r="J45" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K45" s="13" t="n"/>
     </row>
     <row r="46">
@@ -2245,7 +2397,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J46" s="13" t="n"/>
+      <c r="J46" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K46" s="13" t="n"/>
     </row>
     <row r="47">
@@ -2281,7 +2437,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J47" s="13" t="n"/>
+      <c r="J47" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K47" s="13" t="n"/>
     </row>
     <row r="48">
@@ -2321,7 +2481,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J48" s="13" t="n"/>
+      <c r="J48" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K48" s="13" t="n"/>
     </row>
     <row r="49">
@@ -2357,7 +2521,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J49" s="13" t="n"/>
+      <c r="J49" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K49" s="13" t="n"/>
     </row>
     <row r="50">
@@ -2393,7 +2561,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J50" s="13" t="n"/>
+      <c r="J50" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K50" s="13" t="n"/>
     </row>
     <row r="51">
@@ -2429,7 +2601,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J51" s="13" t="n"/>
+      <c r="J51" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K51" s="13" t="n"/>
     </row>
     <row r="52">
@@ -2465,7 +2641,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J52" s="13" t="n"/>
+      <c r="J52" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K52" s="13" t="n"/>
     </row>
     <row r="53">
@@ -2501,7 +2681,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J53" s="13" t="n"/>
+      <c r="J53" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K53" s="13" t="n"/>
     </row>
     <row r="54">
@@ -2541,7 +2725,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J54" s="13" t="n"/>
+      <c r="J54" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K54" s="13" t="n"/>
     </row>
     <row r="55">
@@ -2577,7 +2765,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J55" s="13" t="n"/>
+      <c r="J55" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K55" s="13" t="n"/>
     </row>
     <row r="56">
@@ -2613,7 +2805,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J56" s="13" t="n"/>
+      <c r="J56" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K56" s="13" t="n"/>
     </row>
     <row r="57">
@@ -2653,7 +2849,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J57" s="13" t="n"/>
+      <c r="J57" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K57" s="13" t="n"/>
     </row>
     <row r="58">
@@ -2689,7 +2889,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J58" s="13" t="n"/>
+      <c r="J58" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K58" s="13" t="n"/>
     </row>
     <row r="59">
@@ -2725,7 +2929,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J59" s="13" t="n"/>
+      <c r="J59" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="K59" s="13" t="n"/>
     </row>
     <row r="60">
@@ -2761,7 +2969,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J60" s="13" t="n"/>
+      <c r="J60" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K60" s="13" t="n"/>
     </row>
     <row r="61">
@@ -2797,7 +3009,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J61" s="13" t="n"/>
+      <c r="J61" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K61" s="13" t="n"/>
     </row>
     <row r="62">
@@ -2833,7 +3049,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J62" s="13" t="n"/>
+      <c r="J62" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K62" s="13" t="n"/>
     </row>
     <row r="63">
@@ -2869,7 +3089,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J63" s="13" t="n"/>
+      <c r="J63" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K63" s="13" t="n"/>
     </row>
     <row r="64">
@@ -2909,7 +3133,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J64" s="13" t="n"/>
+      <c r="J64" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K64" s="13" t="n"/>
     </row>
     <row r="65">
@@ -2961,7 +3189,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J66" s="13" t="n"/>
+      <c r="J66" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K66" s="13" t="n"/>
     </row>
     <row r="67">
@@ -2997,7 +3229,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J67" s="13" t="n"/>
+      <c r="J67" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K67" s="13" t="n"/>
     </row>
     <row r="68">
@@ -3033,7 +3269,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J68" s="13" t="n"/>
+      <c r="J68" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K68" s="13" t="n"/>
     </row>
     <row r="69">
@@ -3069,7 +3309,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J69" s="13" t="n"/>
+      <c r="J69" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K69" s="13" t="n"/>
     </row>
     <row r="70">
@@ -3105,7 +3349,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J70" s="13" t="n"/>
+      <c r="J70" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K70" s="13" t="n"/>
     </row>
     <row r="71">
@@ -3141,7 +3389,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J71" s="13" t="n"/>
+      <c r="J71" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K71" s="13" t="n"/>
     </row>
     <row r="72">
@@ -3177,7 +3429,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J72" s="13" t="n"/>
+      <c r="J72" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K72" s="13" t="n"/>
     </row>
     <row r="73">
@@ -3213,7 +3469,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J73" s="13" t="n"/>
+      <c r="J73" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K73" s="13" t="n"/>
     </row>
     <row r="74">
@@ -3249,7 +3509,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J74" s="13" t="n"/>
+      <c r="J74" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K74" s="13" t="n"/>
     </row>
     <row r="75">
@@ -3285,7 +3549,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J75" s="13" t="n"/>
+      <c r="J75" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K75" s="13" t="n"/>
     </row>
     <row r="76">
@@ -3321,7 +3589,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J76" s="13" t="n"/>
+      <c r="J76" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K76" s="13" t="n"/>
     </row>
     <row r="77">
@@ -3357,7 +3629,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J77" s="13" t="n"/>
+      <c r="J77" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K77" s="13" t="n"/>
     </row>
     <row r="78">
@@ -3397,7 +3673,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J78" s="13" t="n"/>
+      <c r="J78" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K78" s="13" t="n"/>
     </row>
     <row r="79">
@@ -3433,7 +3713,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J79" s="13" t="n"/>
+      <c r="J79" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K79" s="13" t="n"/>
     </row>
     <row r="80">
@@ -3469,7 +3753,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J80" s="13" t="n"/>
+      <c r="J80" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K80" s="13" t="n"/>
     </row>
     <row r="81">
@@ -3505,7 +3793,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J81" s="13" t="n"/>
+      <c r="J81" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K81" s="13" t="n"/>
     </row>
     <row r="82">
@@ -3541,7 +3833,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J82" s="13" t="n"/>
+      <c r="J82" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K82" s="13" t="n"/>
     </row>
     <row r="83">
@@ -3597,7 +3893,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J84" s="13" t="n"/>
+      <c r="J84" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K84" s="13" t="n"/>
     </row>
     <row r="85">
@@ -3633,7 +3933,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J85" s="13" t="n"/>
+      <c r="J85" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K85" s="13" t="n"/>
     </row>
     <row r="86">
@@ -3669,7 +3973,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J86" s="13" t="n"/>
+      <c r="J86" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K86" s="13" t="n"/>
     </row>
     <row r="87">
@@ -3705,7 +4013,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J87" s="13" t="n"/>
+      <c r="J87" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K87" s="13" t="n"/>
     </row>
     <row r="88">
@@ -3741,7 +4053,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J88" s="13" t="n"/>
+      <c r="J88" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K88" s="13" t="n"/>
     </row>
     <row r="89">
@@ -3797,7 +4113,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J90" s="13" t="n"/>
+      <c r="J90" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K90" s="13" t="n"/>
     </row>
     <row r="91">
@@ -3833,7 +4153,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J91" s="13" t="n"/>
+      <c r="J91" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="K91" s="13" t="n"/>
     </row>
     <row r="92">
@@ -3869,7 +4193,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J92" s="13" t="n"/>
+      <c r="J92" s="14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="K92" s="13" t="n"/>
     </row>
     <row r="93">
@@ -3905,7 +4233,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J93" s="13" t="n"/>
+      <c r="J93" s="12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="K93" s="13" t="n"/>
     </row>
     <row r="94"/>
@@ -4342,14 +4674,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F19"/>
+  <dimension ref="B2:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
     <col width="92" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -4363,14 +4695,14 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Rep 1: 57   Rep 2: 72   Rep 3: 71   Rep 4: 70 (paper)   Rep 5: 73 / 78     content only /74:  57 · 70 · 69 · 70 · 71</t>
+          <t>Rep 1: 57   Rep 2: 72   Rep 3: 71   Rep 4: 70 (paper)   Rep 5: 73   Rep 6: 72  / 78</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="53" t="inlineStr">
-        <is>
-          <t>Rep 5 is the best score yet, and the first with all four schedules AND a complete balance sheet in the same rep.</t>
+      <c r="B5" s="55" t="inlineStr">
+        <is>
+          <t>Content only, out of 74:  57 · 70 · 69 · 70 · 71 · 70.  Five reps inside a 4-point band - the skeleton has converged.</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4733,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="54" customHeight="1">
+    <row r="9" ht="52" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
         <is>
           <t>1</t>
@@ -4409,213 +4741,214 @@
       </c>
       <c r="C9" s="43" t="inlineStr">
         <is>
+          <t>Rep 6</t>
+        </is>
+      </c>
+      <c r="D9" s="44" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>You started adapting the skeleton to the case</t>
+        </is>
+      </c>
+      <c r="F9" s="30" t="inlineStr">
+        <is>
+          <t>A Costs Schedule driven off an inflation rate, a revolver continuance fee, short-term debt balance and rate. These are not from memory - they are read out of the Larkfield notes. That is a real step past rote recall.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C10" s="43" t="inlineStr">
+        <is>
+          <t>Rep 6</t>
+        </is>
+      </c>
+      <c r="D10" s="44" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>Balance check now carries live formulas</t>
+        </is>
+      </c>
+      <c r="F10" s="30">
+        <f>E69-E87 across all eight columns. First computational content in any skeleton rep, and it is the right cell to put the first formula in.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C11" s="43" t="inlineStr">
+        <is>
+          <t>Rep 4</t>
+        </is>
+      </c>
+      <c r="D11" s="44" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>Revolver line in cash flow financing</t>
+        </is>
+      </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>B113 in financing. Cash flow is 17/17 for the second rep running.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C12" s="43" t="inlineStr">
+        <is>
+          <t>Rep 5</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>REGRESSED</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>Minimum cash balance dropped from assumptions</t>
+        </is>
+      </c>
+      <c r="F12" s="30" t="inlineStr">
+        <is>
+          <t>Present in rep 5, gone now. Note 5 of the Larkfield report gives BOTH the 0.35% commitment fee AND the $60.0m minimum cash covenant - you took the fee and left the covenant. Without a minimum the revolver sweep has nothing to solve against.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="52" customHeight="1">
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C13" s="43" t="inlineStr">
+        <is>
+          <t>Rep 6</t>
+        </is>
+      </c>
+      <c r="D13" s="33" t="inlineStr">
+        <is>
+          <t>NEW MISS</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>No standalone Total Liabilities row</t>
+        </is>
+      </c>
+      <c r="F13" s="30" t="inlineStr">
+        <is>
+          <t>Balance sheet runs Total Current Liabilities, Total Non-Current Liabilities, then straight into equity. Arithmetically fine - Total L&amp;SE can sum the three - but it is a presentation line every real balance sheet has.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="52" customHeight="1">
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C14" s="43" t="inlineStr">
+        <is>
+          <t>Rep 5</t>
+        </is>
+      </c>
+      <c r="D14" s="45" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>Dividends as a % of net income still absent</t>
+        </is>
+      </c>
+      <c r="F14" s="30" t="inlineStr">
+        <is>
+          <t>Gone for two reps now. The Dividends line survives on the income statement, cash flow and equity schedule; only the driver is missing. Larkfield note 7 gives you the payout target of about one third.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C15" s="43" t="inlineStr">
+        <is>
+          <t>Rep 5</t>
+        </is>
+      </c>
+      <c r="D15" s="45" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>Revolver draw and repay formulas not rebuilt</t>
+        </is>
+      </c>
+      <c r="F15" s="30" t="inlineStr">
+        <is>
+          <t>The block is there with Draw, Repayment and Ending rows, but empty. Rep 5 had working logic with a sign error on the ending line - rebuild it WITH the fix: ending = beginning + draw - repayment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52" customHeight="1">
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C16" s="43" t="inlineStr">
+        <is>
           <t>Rep 2</t>
         </is>
       </c>
-      <c r="D9" s="44" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>Income taxes payable on the balance sheet</t>
-        </is>
-      </c>
-      <c r="F9" s="30" t="inlineStr">
-        <is>
-          <t>B73, in current liabilities. Failed three of the first four reps - present in rep 5. This was the big one.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="54" customHeight="1">
-      <c r="B10" s="17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C10" s="43" t="inlineStr">
-        <is>
-          <t>Rep 4</t>
-        </is>
-      </c>
-      <c r="D10" s="44" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="E10" s="17" t="inlineStr">
-        <is>
-          <t>The PP&amp;E chain</t>
-        </is>
-      </c>
-      <c r="F10" s="30" t="inlineStr">
-        <is>
-          <t>Asset schedule back at B196-199 as a proper roll-forward, and the depreciation-as-%-of-PP&amp;E driver back at B10.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="54" customHeight="1">
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C11" s="43" t="inlineStr">
-        <is>
-          <t>Rep 2</t>
-        </is>
-      </c>
-      <c r="D11" s="44" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="E11" s="17" t="inlineStr">
-        <is>
-          <t>Debt schedule</t>
-        </is>
-      </c>
-      <c r="F11" s="30" t="inlineStr">
-        <is>
-          <t>Best version yet: long-term and short-term modelled separately, each with beginning, increase-(repayment), ending, its own rate and its own interest expense line.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="54" customHeight="1">
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C12" s="43" t="inlineStr">
-        <is>
-          <t>Rep 2</t>
-        </is>
-      </c>
-      <c r="D12" s="33" t="inlineStr">
-        <is>
-          <t>BUG</t>
-        </is>
-      </c>
-      <c r="E12" s="17" t="inlineStr">
-        <is>
-          <t>Revolver ending balance ADDS the repayment</t>
-        </is>
-      </c>
-      <c r="F12" s="30">
-        <f>SUM(E178:E180) sums beginning + draw + repayment, but the repayment is computed as a POSITIVE number - so the revolver GROWS when it should shrink. Wrong in 3 of 6 stress cases: begin 40, cash 200, min 140 gives 80 where it should give 0. Fix: make the repayment negative, =-MAX(MIN(E173-E176,E178),0), and keep the SUM.</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="54" customHeight="1">
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C13" s="43" t="inlineStr">
-        <is>
-          <t>Rep 5</t>
-        </is>
-      </c>
-      <c r="D13" s="35" t="inlineStr">
-        <is>
-          <t>NOTE</t>
-        </is>
-      </c>
-      <c r="E13" s="17" t="inlineStr">
-        <is>
-          <t>The draw and repay LOGIC is now correct</t>
-        </is>
-      </c>
-      <c r="F13" s="30">
-        <f>MAX(E176-E173,0) and =MAX(MIN(E173-E176,E178),0). The MIN cap that was missing in rep 2 is there and correct in every stress case. Only the sign on the ending line is wrong.</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="54" customHeight="1">
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C14" s="43" t="inlineStr">
-        <is>
-          <t>Rep 5</t>
-        </is>
-      </c>
-      <c r="D14" s="35" t="inlineStr">
-        <is>
-          <t>NOTE</t>
-        </is>
-      </c>
-      <c r="E14" s="17" t="inlineStr">
-        <is>
-          <t>Your test case hides the bug - again</t>
-        </is>
-      </c>
-      <c r="F14" s="30" t="inlineStr">
-        <is>
-          <t>Cash 120 against a 140 minimum is a DRAW year, so the repayment is zero and the sign error cannot show. Rep 2 had exactly the same blind spot. When you test a sweep, always test a repayment year too.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="54" customHeight="1">
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C15" s="43" t="inlineStr">
-        <is>
-          <t>Rep 5</t>
-        </is>
-      </c>
-      <c r="D15" s="33" t="inlineStr">
-        <is>
-          <t>REGRESSED</t>
-        </is>
-      </c>
-      <c r="E15" s="17" t="inlineStr">
-        <is>
-          <t>Dividends as a % of net income dropped from assumptions</t>
-        </is>
-      </c>
-      <c r="F15" s="30" t="inlineStr">
-        <is>
-          <t>Present in reps 1 through 4. The Dividends line is still on the income statement and in both the cash flow and the equity schedule - only the driver went.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="54" customHeight="1">
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C16" s="43" t="inlineStr">
-        <is>
-          <t>Rep 4</t>
-        </is>
-      </c>
-      <c r="D16" s="33" t="inlineStr">
-        <is>
-          <t>REGRESSED</t>
+      <c r="D16" s="45" t="inlineStr">
+        <is>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="E16" s="17" t="inlineStr">
         <is>
-          <t>No revolver line in cash flow financing</t>
+          <t>No colour convention</t>
         </is>
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>You had it in rep 4. Financing is back to debt, equity and dividends only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="54" customHeight="1">
+          <t>All 257 populated cells still default theme font. Six reps. This one costs nothing and you keep skipping it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="52" customHeight="1">
       <c r="B17" s="17" t="inlineStr">
         <is>
           <t>9</t>
@@ -4623,7 +4956,7 @@
       </c>
       <c r="C17" s="43" t="inlineStr">
         <is>
-          <t>Rep 2</t>
+          <t>Rep 3</t>
         </is>
       </c>
       <c r="D17" s="45" t="inlineStr">
@@ -4633,16 +4966,12 @@
       </c>
       <c r="E17" s="17" t="inlineStr">
         <is>
-          <t>No colour convention</t>
-        </is>
-      </c>
-      <c r="F17" s="30" t="inlineStr">
-        <is>
-          <t>All 230 populated cells still default theme font. This is the last easy structural win.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="54" customHeight="1">
+          <t>No actual vs projected markers</t>
+        </is>
+      </c>
+      <c r="F17" s="30" t="inlineStr"/>
+    </row>
+    <row r="18" ht="52" customHeight="1">
       <c r="B18" s="17" t="inlineStr">
         <is>
           <t>10</t>
@@ -4653,42 +4982,64 @@
           <t>Rep 3</t>
         </is>
       </c>
-      <c r="D18" s="45" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="D18" s="33" t="inlineStr">
+        <is>
+          <t>OVERDUE</t>
         </is>
       </c>
       <c r="E18" s="17" t="inlineStr">
         <is>
-          <t>No actual vs projected markers</t>
-        </is>
-      </c>
-      <c r="F18" s="30" t="inlineStr"/>
-    </row>
-    <row r="19" ht="54" customHeight="1">
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C19" s="43" t="inlineStr">
-        <is>
-          <t>Rep 3</t>
-        </is>
-      </c>
-      <c r="D19" s="44" t="inlineStr">
-        <is>
-          <t>CLOSING</t>
-        </is>
-      </c>
-      <c r="E19" s="17" t="inlineStr">
-        <is>
-          <t>Assumption values</t>
-        </is>
-      </c>
-      <c r="F19" s="30" t="inlineStr">
-        <is>
-          <t>Five reps, no numbers. Resolved now - the fake report is the input for the next rep.</t>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F18" s="30" t="inlineStr">
+        <is>
+          <t>Six skeleton reps, still zero values. The Larkfield report has been ready since the last rep. This is now the only thing standing between you and a model that closes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="56" t="inlineStr">
+        <is>
+          <t>THE CALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="31" t="inlineStr">
+        <is>
+          <t>Rep 1 to 2 gained 13 points. Reps 2 through 6 have sat between 69 and 71 out of 74.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="31" t="inlineStr">
+        <is>
+          <t>The skeleton is not getting better any more - it is finished, and the remaining misses are</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="31" t="inlineStr">
+        <is>
+          <t>small enough that a three-minute closing sweep catches them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="31" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>Stop drilling the skeleton. Next rep is numbers: type the Larkfield historicals in, compute the</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>historical ratios, and set the assumptions. That is the Day 2 and Day 3 layer, five days overdue.</t>
         </is>
       </c>
     </row>
@@ -4979,9 +5330,9 @@
           <t>Day 3</t>
         </is>
       </c>
-      <c r="C10" s="54" t="inlineStr">
-        <is>
-          <t>NEXT</t>
+      <c r="C10" s="57" t="inlineStr">
+        <is>
+          <t>DO NEXT</t>
         </is>
       </c>
       <c r="D10" s="17" t="inlineStr">

</xml_diff>

<commit_message>
Close the skeleton phase and open the full-build ladder
Six skeleton reps converged between 70 and 73 of 78, and the first
complete model would have scored full marks on that scorecard while
carrying two wrong figures. Completeness has stopped being the useful
measure, so the ladder now counts full builds and the goal becomes
correctness.

Replaces the day-based ladder with eight builds, starting with repairing
the current model in place rather than rebuilding it, and adds a
four-step verification sweep to run before any build is called finished.
The first step, selecting constants across the forecast columns, would
have surfaced the hardcoded cash roll-forward immediately.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UX5HPwj2AEakAb4LMEQ7Bv
</commit_message>
<xml_diff>
--- a/learning/model-practice/Day_2_scorecard_and_ladder.xlsx
+++ b/learning/model-practice/Day_2_scorecard_and_ladder.xlsx
@@ -216,7 +216,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -253,6 +253,11 @@
         <fgColor rgb="FFF0F0F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF6DA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -280,7 +285,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -383,6 +388,20 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4240,7 +4259,6 @@
       </c>
       <c r="K93" s="13" t="n"/>
     </row>
-    <row r="94"/>
     <row r="95">
       <c r="B95" s="3" t="inlineStr">
         <is>
@@ -5227,355 +5245,401 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E29"/>
+  <dimension ref="B2:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="86" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Fourteen-Day Ladder</t>
+          <t>Phase 2 — Full Builds</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>One rule: every day you rebuild everything from the previous days from a blank sheet FIRST, then add that day's new layer.</t>
+          <t>The skeleton phase is closed. Six reps, converged at 70-73 of 78. Nothing left to learn there.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>The rebuild is the rep. The new layer is the lesson. Skipping the rebuild turns this back into passive tutorial-following.</t>
+      <c r="B4" s="58" t="inlineStr">
+        <is>
+          <t>From here the unit of practice is a COMPLETE MODEL, and the thing being tested is correctness, not completeness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="52" t="inlineStr">
+        <is>
+          <t>WHY THE MEASURE HAS TO CHANGE</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>Your first full model scored 78/78 on the old scorecard - every line present, balance check zero in all eight columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="31" t="inlineStr">
+        <is>
+          <t>It also had two wrong numbers in it. The scorecard cannot see those, and neither can the balance check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>Completeness was the right measure while lines were going missing. It is the wrong measure now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Layer</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>What you actually do</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>Day 1</t>
-        </is>
-      </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Why it is next</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="B13" s="59" t="inlineStr">
+        <is>
+          <t>Build 1</t>
+        </is>
+      </c>
+      <c r="C13" s="60" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
-        <is>
-          <t>Blind skeleton</t>
-        </is>
-      </c>
-      <c r="E8" s="30" t="inlineStr">
-        <is>
-          <t>Labels only, no numbers. Scored 73% on the Scorecard tab.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="44" customHeight="1">
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>Day 2</t>
-        </is>
-      </c>
-      <c r="C9" s="29" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D9" s="17" t="inlineStr">
-        <is>
-          <t>Periods + assumptions</t>
-        </is>
-      </c>
-      <c r="E9" s="30" t="inlineStr">
-        <is>
-          <t>Skeleton is essentially automatic: 73/78, all four schedules, complete balance sheet, working MIN/MAX draw and repay logic. Move to Day 3 - put real numbers in from the Larkfield report.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="B10" s="17" t="inlineStr">
-        <is>
-          <t>Day 3</t>
-        </is>
-      </c>
-      <c r="C10" s="57" t="inlineStr">
+      <c r="D13" s="59" t="inlineStr">
+        <is>
+          <t>First close on Larkfield</t>
+        </is>
+      </c>
+      <c r="E13" s="61" t="inlineStr">
+        <is>
+          <t>Complete model, balances to 2.3e-13. Two critical errors, two dormant, four structural. Reviewed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="B14" s="62" t="inlineStr">
+        <is>
+          <t>Build 2</t>
+        </is>
+      </c>
+      <c r="C14" s="63" t="inlineStr">
         <is>
           <t>DO NEXT</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
-        <is>
-          <t>Income statement</t>
-        </is>
-      </c>
-      <c r="E10" s="30" t="inlineStr">
-        <is>
-          <t>Rebuild, then drive revenue through to net income with formulas. Every line references an assumption cell - no number typed inside a formula.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>Day 4</t>
-        </is>
-      </c>
-      <c r="C11" s="29" t="inlineStr"/>
-      <c r="D11" s="17" t="inlineStr">
-        <is>
-          <t>PP&amp;E + working capital schedules</t>
-        </is>
-      </c>
-      <c r="E11" s="30" t="inlineStr">
-        <is>
-          <t>Rebuild, then both schedules as proper roll-forwards. This is the day the word 'schedule' should stop feeling abstract.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>Day 5</t>
-        </is>
-      </c>
-      <c r="C12" s="29" t="inlineStr"/>
-      <c r="D12" s="17" t="inlineStr">
-        <is>
-          <t>Balance sheet + the check row</t>
-        </is>
-      </c>
-      <c r="E12" s="30" t="inlineStr">
-        <is>
-          <t>Rebuild, then the balance sheet with the check row at the bottom. Expect it NOT to balance - you have no cash flow statement yet. That is correct.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>Day 6</t>
-        </is>
-      </c>
-      <c r="C13" s="29" t="inlineStr"/>
-      <c r="D13" s="17" t="inlineStr">
-        <is>
-          <t>Cash flow statement - first close</t>
-        </is>
-      </c>
-      <c r="E13" s="30" t="inlineStr">
-        <is>
-          <t>Rebuild, then the CFS. Chase the check row to zero. This is the day the model becomes a model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>Day 7</t>
-        </is>
-      </c>
-      <c r="C14" s="29" t="inlineStr"/>
-      <c r="D14" s="17" t="inlineStr">
-        <is>
-          <t>Full rebuild, timed</t>
-        </is>
-      </c>
-      <c r="E14" s="30" t="inlineStr">
-        <is>
-          <t>Everything from blank, on the clock. Write the time down. This is your baseline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
+      <c r="D14" s="62" t="inlineStr">
+        <is>
+          <t>Fix the six findings IN PLACE</t>
+        </is>
+      </c>
+      <c r="E14" s="64" t="inlineStr">
+        <is>
+          <t>Do not rebuild. Repair. Relink rows 248-250, move depreciation to opening PP&amp;E, rebuild and connect the revolver, repoint the backwards links, swap the goodwill and intangibles labels. Fixing is a separate skill from building and you have never practised it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>Day 8</t>
-        </is>
-      </c>
-      <c r="C15" s="29" t="inlineStr"/>
+          <t>Build 3</t>
+        </is>
+      </c>
+      <c r="C15" s="57" t="inlineStr"/>
       <c r="D15" s="17" t="inlineStr">
         <is>
-          <t>Debt schedule</t>
+          <t>Larkfield from blank, WITH numbers, timed</t>
         </is>
       </c>
       <c r="E15" s="30" t="inlineStr">
         <is>
-          <t>Rebuild, then a real debt schedule. Interest on the OPENING balance for now - no circularity yet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
+          <t>Everything, empty workbook, on the clock. Expect three to four hours. Do not chase a target - just record the number. This is your real baseline; the 44 minutes was only a skeleton.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>Day 9</t>
-        </is>
-      </c>
-      <c r="C16" s="29" t="inlineStr"/>
+          <t>Build 4</t>
+        </is>
+      </c>
+      <c r="C16" s="57" t="inlineStr"/>
       <c r="D16" s="17" t="inlineStr">
         <is>
-          <t>Full rebuild with debt</t>
+          <t>Larkfield from blank again</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
         <is>
-          <t>No new layer. Just do the whole thing again and beat Day 7's time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
+          <t>No new material. Beat build 3's time and hit zero findings on your own verification sweep before you look at anything else.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>Day 10</t>
-        </is>
-      </c>
-      <c r="C17" s="29" t="inlineStr"/>
+          <t>Build 5</t>
+        </is>
+      </c>
+      <c r="C17" s="57" t="inlineStr"/>
       <c r="D17" s="17" t="inlineStr">
         <is>
-          <t>Equity schedule + dividends</t>
+          <t>Larkfield from blank, under 2h30</t>
         </is>
       </c>
       <c r="E17" s="30" t="inlineStr">
         <is>
-          <t>Rebuild, then the equity roll-forward. Make sure dividends leave through financing - that was a Day 1 miss.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
+          <t>By now the sequence should be automatic and the time should be going into judgement, not recall.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>Day 11</t>
-        </is>
-      </c>
-      <c r="C18" s="29" t="inlineStr"/>
+          <t>Build 6</t>
+        </is>
+      </c>
+      <c r="C18" s="57" t="inlineStr"/>
       <c r="D18" s="17" t="inlineStr">
         <is>
-          <t>Revolver + MIN/MAX sweep</t>
+          <t>Break it on purpose</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Rebuild, then the minimum cash balance and the sweep. Drill 3 on the drills page until the logic is automatic BEFORE you build it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
+          <t>Take a finished build. Set revenue growth to -5% for three years. The revolver must draw, the balance check must hold, and nothing may go negative that shouldn't. Then have someone break one link at random and time yourself finding it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>Day 12</t>
-        </is>
-      </c>
-      <c r="C19" s="29" t="inlineStr"/>
+          <t>Build 7</t>
+        </is>
+      </c>
+      <c r="C19" s="57" t="inlineStr"/>
       <c r="D19" s="17" t="inlineStr">
         <is>
-          <t>Switch to average-balance interest</t>
+          <t>Larkfield from blank, under 2h</t>
         </is>
       </c>
       <c r="E19" s="30" t="inlineStr">
         <is>
-          <t>Rebuild, then flip interest to the average method and turn on iterative calculation. Add a circuit-breaker switch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
+          <t>This is the competence benchmark from the program. Same company, seventh time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Day 13</t>
-        </is>
-      </c>
-      <c r="C20" s="29" t="inlineStr"/>
+          <t>Build 8</t>
+        </is>
+      </c>
+      <c r="C20" s="57" t="inlineStr"/>
       <c r="D20" s="17" t="inlineStr">
         <is>
-          <t>Full rebuild, timed</t>
+          <t>A REAL company</t>
         </is>
       </c>
       <c r="E20" s="30" t="inlineStr">
         <is>
-          <t>Everything, from blank, on the clock. Compare against Day 7.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="17" t="inlineStr">
-        <is>
-          <t>Day 14</t>
-        </is>
-      </c>
-      <c r="C21" s="29" t="inlineStr"/>
-      <c r="D21" s="17" t="inlineStr">
-        <is>
-          <t>New company</t>
-        </is>
-      </c>
-      <c r="E21" s="30" t="inlineStr">
-        <is>
-          <t>Same model, different business. This is where the skill stops being one memorised spreadsheet and starts being a skill.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
+          <t>Pull a 10-K from SEC EDGAR. Pick something boring - a grocer, a distributor, a single-product manufacturer. Everything changes except the model, which is the whole point.</t>
+        </is>
+      </c>
+    </row>
     <row r="23">
-      <c r="B23" s="23" t="inlineStr">
-        <is>
-          <t>Every day, before the build:</t>
+      <c r="B23" s="56" t="inlineStr">
+        <is>
+          <t>THE NEW VERIFICATION SWEEP — run all four before calling any build finished</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="31" t="inlineStr">
-        <is>
-          <t>5 minutes of drills, then the blank skeleton from memory.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="23" t="inlineStr">
-        <is>
-          <t>Every day, after the build:</t>
+      <c r="B24" s="36" t="inlineStr">
+        <is>
+          <t>The balance check is now necessary but nowhere near sufficient. These four catch what it cannot.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="31" t="inlineStr">
-        <is>
-          <t>One line in the rep log - what broke, and how many minutes it cost.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>How</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>What it catches</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="58" customHeight="1">
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>Hunt every hardcode in the forecast</t>
+        </is>
+      </c>
+      <c r="D27" s="30" t="inlineStr">
+        <is>
+          <t>Select the forecast columns only. F5 → Special → Constants → OK. Every hardcoded cell lights up.</t>
+        </is>
+      </c>
+      <c r="E27" s="65" t="inlineStr">
+        <is>
+          <t>THIS WOULD HAVE CAUGHT FINDING 1 IN FIVE SECONDS. Rows 248-250 would have selected immediately. Nothing in a forecast column should be a typed number - every value is a formula off an assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="58" customHeight="1">
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>Trace one line end to end</t>
+        </is>
+      </c>
+      <c r="D28" s="30" t="inlineStr">
+        <is>
+          <t>Pick depreciation. Follow it: asset schedule → income statement → cash flow add-back → PP&amp;E closing balance. Check the same number appears in all four and with the right sign.</t>
+        </is>
+      </c>
+      <c r="E28" s="65" t="inlineStr">
+        <is>
+          <t>Broken links, sign errors, and a driver applied to the wrong balance - which is finding 2 exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="58" customHeight="1">
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>Recompute the forecast ratios</t>
+        </is>
+      </c>
+      <c r="D29" s="30" t="inlineStr">
+        <is>
+          <t>Calculate the ratios OUT of your forecast the same way you calculated them out of history. Compare against the assumptions you set.</t>
+        </is>
+      </c>
+      <c r="E29" s="65" t="inlineStr">
+        <is>
+          <t>Anywhere the model is not doing what you told it to. If you set 13% depreciation and the forecast implies 13.6%, you are charging it on the wrong base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="58" customHeight="1">
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>Stress it</t>
+        </is>
+      </c>
+      <c r="D30" s="30" t="inlineStr">
+        <is>
+          <t>Revenue growth to -5%. Then minimum cash to 200.</t>
+        </is>
+      </c>
+      <c r="E30" s="65" t="inlineStr">
+        <is>
+          <t>Dormant logic. Your revolver formula is wrong in four of six cases and you would never know, because cash never falls far enough to fire it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>WHERE THIS ENDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="23" t="inlineStr">
+        <is>
+          <t>Eight full builds gets you to the competence benchmark: a simple company, blank sheet, under two hours, balanced,</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="23" t="inlineStr">
+        <is>
+          <t>with a working debt schedule and revolver. That is the level the training shops call 'can do the job'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="31" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="31" t="inlineStr">
+        <is>
+          <t>After that the ladder is: 90-minute cuts, then a genuinely messy filing, then interleaving companies at random.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="31" t="inlineStr">
+        <is>
+          <t>But none of that matters until build 8. Do not skip ahead - the reps ARE the method.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>